<commit_message>
update use local YOLO แทน roboflow
</commit_message>
<xml_diff>
--- a/insect_analysis_history.xlsx
+++ b/insect_analysis_history.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="49">
   <si>
     <t>วันที่ตรวจ</t>
   </si>
@@ -46,6 +46,9 @@
     <t>จำนวนแมลงอื่นๆ</t>
   </si>
   <si>
+    <t>รูปภาพ</t>
+  </si>
+  <si>
     <t>2026-03-09</t>
   </si>
   <si>
@@ -55,6 +58,12 @@
     <t>2026-03-02</t>
   </si>
   <si>
+    <t>2026-04-20</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
     <t>11:45:46</t>
   </si>
   <si>
@@ -70,6 +79,39 @@
     <t>16:17:24</t>
   </si>
   <si>
+    <t>15:16:41</t>
+  </si>
+  <si>
+    <t>15:18:07</t>
+  </si>
+  <si>
+    <t>15:18:50</t>
+  </si>
+  <si>
+    <t>15:30:55</t>
+  </si>
+  <si>
+    <t>16:01:35</t>
+  </si>
+  <si>
+    <t>16:47:34</t>
+  </si>
+  <si>
+    <t>16:51:16</t>
+  </si>
+  <si>
+    <t>08:50:28</t>
+  </si>
+  <si>
+    <t>08:50:52</t>
+  </si>
+  <si>
+    <t>08:51:28</t>
+  </si>
+  <si>
+    <t>08:54:36</t>
+  </si>
+  <si>
     <t>SB</t>
   </si>
   <si>
@@ -91,6 +133,12 @@
     <t>เครื่องที่ 2</t>
   </si>
   <si>
+    <t>ห้อง Mix SP</t>
+  </si>
+  <si>
+    <t>ห้อง Pack SP</t>
+  </si>
+  <si>
     <t>ฺฤฆ</t>
   </si>
   <si>
@@ -100,10 +148,19 @@
     <t>Pratcahyaw</t>
   </si>
   <si>
+    <t>BASS</t>
+  </si>
+  <si>
     <t>หกห</t>
   </si>
   <si>
     <t>ทดสอบ</t>
+  </si>
+  <si>
+    <t>/9j/4AAQSkZJRgABAQAAAQABAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCAQ0BfEDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwDstchiuvjJosE0EcyfY5SUkUMPrg13R0DRiDnSbE5GD/o6c/pXEakSPjdo+TwbGXH516RU9WZwW5lDwzoQ6aLpw/7dU/wqQeH9GU5Gk2IPtbp/hWlRTsi7Izv7C0jOf7Lss/8AXuv+FL/Yek/9Auy/8B1/wrQoosFjOOh6T0/suy/8B1/wpf7E0sjH9mWeP+uC/wCFaPFFFgsZp0HSHOW0uyP1t1/wpP8AhH9Gzn+ybH/wHT/CtKiiyCyM8aFpA6aVZD/t3X/Cl/sTSf8AoFWP/gOv+FX6KYyh/Ymlf9Ayy/78L/hQdE0s9dNsz9YF/wAK0KSlYDy260fTP+F26fbjTrQQ/wBlySGMQLgnPXGOtehLomlgfLptmB7QL/hXD3bBvjzp645XSpD+tekUrIiKRROj6ZjB060x6eQv+FJ/Ymkn/mGWf/gOv+FX6Kdi7Gf/AGHpP/QLsv8AwHX/AApn/COaJ/0B9P8A/AVP8K1OKKLCsZY8O6KowNH08D0Fsn+FH/CPaLkn+x7DJ7/Zk/wrUpKLBZGb/wAI/ov/AECLD/wGT/Cmnw1oZGDo2nH62qf4Vq0UWCyMb/hFPDv/AEAdL/8AAOP/AAobwn4dbltB0s/Wzj/wrYpaLBZGJ/wiPhw4zoGlcf8ATlH/AIUDwj4bB3Dw/pQPr9ij/wAK26KLBZHksPhzRG+NN3Ztounta/2UkohNqmzcXIJxjGeOtd1/whHhT/oWdG/8AIv8K5m1J/4XxfDr/wASiP8AD5jXotCRMUjn/wDhB/CeMf8ACMaN/wCAMX+FIfAnhMkk+GtI5/6co/8ACuioosVZHN/8IB4P/wChY0j/AMA4/wDCmn4feED/AMyxpP4WiD+ldNRRYLI5Vvhv4MY5PhrTc+0AFN/4Vp4LH/Mtaf8A9+q6uinYLI5A/C7wSf8AmW7L/vk/40w/CnwOevhy0/AsP612VFKwWRxZ+E/gVv8AmXbYfRnH9aY3wi8COOfD0PHpNKP5NXb0U7BZHC/8Kd8Af9C7H/3/AJv/AIqmt8G/AR/5gCD6Ty//ABVd5RQFjwrw98NfC2ofELxTpk9gWsrExCCLzmG3cgJ5znqa7Nvgn4Fb/mFSD6XD/wCNR+EW/wCLueNwOmbf/wBFLXo1JImKVjzv/hSXgfjGmzDHpcP/AI0h+CXgs/8ALpdD/t5avRaWixVkecD4I+DFORbXgPqLlqUfBjwzG26GbV4j6x3pFei0UWDlR52fg5ofbVdfH0vz/hSL8ItOjGE8Q+I1+moMK9GpKLC5Ued/8Klsh08SeJR/3EWoPwpjGPJ8WeJ4sf8AUQavRKKLIOVHnrfDG5JO3xx4pX/uIP8A403/AIVjfA5Xx34n/G9Y/wBa9EoosHIjzs/DfWV/1XxA8QKvo0m79SaRvhvreDs+IWvg+75/rXotFFg5EeJeAtG8U+LfDx1Obx1q1sRcSQhEwwIXvk10zeA/F6keV8RdRI7+ZbpTfgcd3w3hz94XU2frmvSaEtBKKsecHwX4537l+IVx7Zs4/wCWKd/wh/j3/ooL/wDgDF/hXo1JRYfKjzr/AIRDx8M4+IDfjYxf4Ug8JfEMf8z4h+tjH/hXo9JiiwcqPOf+EX+JCj5fHFs3+9Yr/hTF8O/E+M/8jhp0g/2rL/AV6TRQHKjzo6H8Tx/zNWlH/tzpDpHxSVfl8SaM597MivRqKYcp5z9g+KwHGsaET/17t/jSfZviwpH+n+H2/wC2Lf416PRQHKedeV8V8f8AHz4e/wC/T/41ieJfEnxN8K2MF5ef2FNFLcJbgRRvnc3TvXr9eb/GlmHhHTyo5Gq25H5mkDVh+/4rqc+R4fcem5hQbn4rA/8AIO0Aj/ru1ejCiiwcp5yL34qgc6XoR+k7Ug1H4qLndomit9LkivR8UUWDl8zzkav8UEG9/DmkuM/dW8IP8qX/AISH4k5/5E+w/wDA7/61eifjQfrQHL5nnh8R/EcH/kTLIj2v/wD61N/4Sf4jjr4Jtj9L4f4V6NRTDl8zzj/hKviIv3vA0Tf7t6Kd/wAJX8QQP+RFjJ/6/h/hXon40fjSDl8zzo+MPiADj/hAfx+2rigeMPH2/DeAG2+ovVr0aiiwW8zzpvGnjVD83gC6/wCA3aGs+x+K2uancXdvZ+Cb2aa0by51Ey/u29DXqleb/DXd/wAJV455G3+1Bx/wGgTT7jl8feKz1+H+o/8Af9KcfHnisHB+H+o/9/4/8a9EpaB2fc86/wCFgeJkHz+ANUGOuJoz/WgfEfW8c+Adaz7Fa9FooCz7nnZ+I2s8Z8Ba3+af400/EvVQMnwHrnHXha9GophZ9zzkfE3Uf4vA2uj6RigfFC+xn/hB9f4/6ZCvRqKQWfc85HxQu+M+CPEAzz/qaafipcg8+CvEP/fivSKKYWfc87b4oyqMnwf4h/8AAU00/FUgc+EfEQ/7dDXo1FAWfc8um+NFjaSxR3nh7W7ZpW2xiW3wXPoB3NT/APC3I+3hTxCc9P8AQ25o+JKeZ4y+H8eOuqlvy2mvScUtRWfc85/4WwuP+RS8SZ/68moHxZTHzeFPES/WyavR8UYpjs+55yPi1bnj/hF/EOfT7C1B+LloBz4b8QjnvYtXo2KTA9KAs+55yfi7aDGfDfiDn/pyaj/hbtrnnw14hH/bi1ejbR6UbR6UCs+55yfi5bZ/5FjxF7f6C1B+LtqvXwz4hH1sWr0fA9KTaPSgdn3PNz8X7Lt4c8QEev2JuaU/GDTx/wAy/r+fT7E1ej7R6UbR/dH5UBZ9zzhPjBYHk+HtfA/68mNNl+MemQI0kmg66sajLM9mQAPU16TtX+6PyrnvHOE8B+IHIHGnz9v+mZo1FZ9zlLf4zabeQia20HXJ426PFaFgfxFSn4v2QOP+Ec8QZ/68Wrd+G0Qj+HOgjHP2Ra6raPSkOzPOf+Fv2WM/8I54g/8AAFqX/hblt28M+If/AABavRdo9BRgelMLPuedn4tWwJH/AAjPiHj/AKcWpR8V4CP+RX8Q/wDgC1eh49qXFAWfc87/AOFrQ4/5FbxF/wCALUh+K8QJH/CK+I//AABavRcUCgLPuedf8LXT/oVPEWfeyakPxYixk+FfEQ/7cmr0YijAoCzPOh8VozjHhXxEf+3JqRviuqHB8JeIuf8ApzNejYoxQFn3POR8VwWwPCPiL6/YzVeH4x2V1czW1t4c1yaaE4kSO3JKH39K9Nrzn4b/AL3xR44nHRtV25+iigWvcP8Aha2CceEfERx/05tUn/C0yUz/AMIj4h9/9DNeh0UDs+552vxRlf7ng7xCfrbYpT8T7jOF8GeICf8Ar3r0OigLPuedf8LQuySP+EK8QZH/AEwFO/4Wdecf8UV4g5/6YivQ6KAs+556fiZeqT/xRPiDHr5IpU+Jly3Twb4gz7wV6DRQFn3PPT8S77nHgnXzgZ/1Ipn/AAs3UD93wNrx/wC2YFei0d6As+553/wsvU8ZHgXXj/wFaP8AhZWrZ48B67+Sf416JRQFn3PLrj4vXFrqFrYT+C9YS8us+RCSu58dcVf/AOFj6znH/CAa5+cf+NQeJFEnxx8GL3S1u3P/AHwa9JHSkCPPm+Ietj/mQNb/AO+o/wDGmn4g+IVx/wAW/wBY5/6ap/jXodFMdmedH4g+Je3w+1b/AL+p/jR/wnvio8D4e6l+M8f+Nei4ooFZnnX/AAnPjDt8PdQ/8CIv8af/AMJt4yzj/hXl/j/r5i/xr0Kigdjz3/hNvGP/AET2/wD/AAJi/wAaQ+N/GIOB8Pr/AD/18xf416HRQFjzo+NfGYz/AMW+vP8AwKj/AMaT/hOPGudv/Cvbv/wKSvRqKBWfc86/4TXxtnj4e3eP+vqP/Gquq/EnxNoenS6hqPge4t7WPG52u4zjJwOlenVwfxiGfhxfAnG6WEf+RBQDTRUi8c+M54lli+H90UcAqftUfI/OpP8AhNPG/wD0T26/8C4/8a7rT126dar6QqP0FWqBo87/AOEz8cf9E+ufxvI/8acPGPjhv+afzA+94lehUUCt5nn3/CYeOc4/4QCX/wADUpR4u8c7gD4Bk57/AG1OK9A/GigdvM8//wCEw8a5I/4QGf8A8DEph8ZeNh/zT66P0vI/8a9DooCx53/wmfjc/wDNPrr/AMC4/wDGlHjHxv8A9E/uf/AyP/GvQ6KAseenxl42A/5J/cZ/6/EpF8Z+ND1+H13/AOBUf+Neh0UBY84uPHXi+1glnm8A3aRRKXdzdR4AAyT1qtpfxI8T61p8Ooad4Fu7i0mBMcq3MYDYOD1PqK7vxISPC+q/9eU3/oBrnvhIMfC3QsH/AJYsf/IjUhdbFQ+NPGGBj4e3+e/+kxf408eNPF2Ofh9qGf8Ar5i/xrvqKY7Hn/8Awm3i3t8PtQ/G4i/xpD438YA/8k9v/wDwJi/xr0GikFjz0+N/GPb4eX//AIExf40o8beMO/w81D/wJi/xr0GimFjz8+OPFCgZ+H2p5/6+Iv8AGov+E/8AFGMn4fapg9P30f8AjXotFIVjzr/hYHic9Ph7qv8A3+j/AMaUePPFZ6fD3Uv+/wDH/jXomKKYWZ56PHPiw4x8PdSz73EX+NO/4Tbxbnn4e6jj/r5i/wAa9ApDSHY8y0/4paprEVw+neCdTuFt5TDKRLH8rjqvXqKvf8J14lYZj+H+rH/eniH9ag+D2f7H8Q8gj+3rvGP+A16OKFcS1PPD8QPEoOD8PtWz/wBdY/8AGlHj7xIevw+1b2/fRf416FRRqOx5+vjvxMx/5J9q3/f6L/GpG8ceI1GT8PtY/wC/0P8AjXeUUBY4H/hP9cwT/wAK/wBb4H/PSL/Gov8AhZGs/wDQga5+cf8AjXodFAHnn/CxdbJ4+H+t/i0f+NPHj/XyOPh/rOfeSP8Axr0CigLHB/8ACe67tyfAGs/9/Iv8ab/wsHWs/wDIg63/AN9x/wCNd7RQFmcEfiDrIHPgLXP++o/8a1PCXjEeKJtQt30u4064sHRJYbhgWywyOntXU1wHgj/kf/HY/wCnyD/0VR1Fqj0GikopjPNr75/jhpfOQunycY6c16TXmsnzfHi2x0GmMf1r0qkt2TAKWkpaZYlFFFABRRS0AFJS0UAFJS0UAJRRRQB5xK2749Wy/wBzRyfzY16PXmsf7z4/yHH3NHA/8eNelUkTEWkpaSmUFLRSUALRRRQAUlLRQAlLRRQAUUUlAHnNiwf48an/ALOkxD/x416NXm2mjd8eNYYZO3S4v516TSRMRaKSimUFLRSUALRRSUALSUtFACUUUtACUGlpKAPOfB4A+LPjjBz80H/opa9GrzbwUxb4p+Oc9fOh/wDRYr0mkiY7BRS0UygopKWgBKKWigAooooAKSlpKAFpDRSMdqk+goA84+COT8OYpP791M3616RXmvwLH/Fs7b/r4l/nXpXagS2FooooGFFJS0AJRRS0AJS0UUAJS0UlABXnHxmXPhjSj3Gr2vH4mvR685+MDD+x9CQ9G1q1z/31QJno1FFFAxaKSigAooooAKKKWgBKWiigBKWiigBO1eb/AAyYN4j8csBj/ibY/SvSO1eb/C879b8byYxnWWH5DFAup6TRRRQMKKKKACikooAKWkpaACkpaKACkpaSgDzf4gEn4ifD5e326Y/+OivSK838aL53xX8BQ+ktxJ+UZP8ASvSKQhaKKKYxKKWigBKWiigAooooAKSlpKACuY+IvHw48RHOP+JfN/6Ca6euR+J7bfhp4hIP/LmwoE9i34AGPAOhD/pzj/lXR1g+CV2eB9EH/TlF/wCgit6gYUtJS0AFJRRQAUtJS0AFFFJQAtJRRQAV518LPnuPFz9m1qX/ANBWvRa89+FSjyfEsndtam/ktBL3R6FS0lLQUFFJRQAUUUUALSUUtACUUUUAFFFFAHnWs7G+Ofhvj510y4OfzH+NeiDgV51qR3fHvRlHVdFlJ/7+GvRRQTHqLRRRQUFFFHNABmjNFGKACjvRRQAUUUUAFcB8Yv8AkndyB/z8wf8Ao0V39ee/GUgfD6QZ63lv/wCjRQJ7HdWYxZQf7g/lViobT/jzg/3B/KpqBoKWkzRQAUtJS0AFJRRQAUUUUAFFFFAGZ4h/5FrVP+vOb/0A1z3wlBHwv0LP/PFv/RjV0HiQ48MasR1FlN/6Aa5/4TMW+F+gnGP3B/8AQ2oJ6naUtJS0FCUUUUAFLSUUAFFFFABRRRQAUhooNAHnPweA/sTX9vA/t67wP++a9Hrzb4Nsp0TX9pyv9uXRH0+WvSRSWwo7BRzRRTGA60mCe9LRQAUUUUALSGiigApaQUUAHauC8F5/4T/xxwB/pUHT/rlXe9q4DwWT/wALC8cg/wDP1B3/AOmQpdSX0PQKKKKZR5lFlvj03oul/wBTXpleaWmD8drvvjTF6duTXpdJdSIbBRRRTLClpKWgBKKKWgApKWkoAWiiigApKWkNAHm9rz8e7vGPl0iMH/vo16RXm1qP+L93hB/5hMef++jXpNJEx2FopKKZQtFJS0AFJS0UAJRS0lABRS0UAJRS0lAHm2jsf+F66+O39mw/zr0mvOtE+b44eIzj7umwD9a9FpImItJS0lMoKWiigAooooAKKKKAEopaKAEoNFB4oA858Fc/E/xywxjz4R/5DFejV5x4KjMfxP8AHSg5Xz4T+JjB/rXo9JEx2FoooplCUUtFABRRRQAUlLRQAUUlFABTW5U56U+o5QTGwXrjigTPOvgac/DG0PrPL/OvSK83+Box8MrU+s8v869IoQLYWiiigYUUUUAJRS0UAFJRRQAtJRRQAV5r8Zcto2hIM5bWLcD869Krzr4rjefCUR6PrtsD/wB9ihiex6KKWkFLQMSilooAKSiigAopaKAEpaKKACkpaSgANeb/AAqG6bxdJ3OuT/oTXo+a85+EZ3Q+KH/va5cn/wAeNAup6RRRSUDCiiloAKKKKAEpaKKACiiigApKWkPSgDzrxPz8Z/Aw9EvP/RL16LXnHiI7/jh4NX+5a3b/APkNhXo9ISFpKWimMKSlooAKKSloAKKKKAEooooAK434rNt+F+vn/p2x/wCPCuyrifi42z4Wa8cdYUH5yKKBPY3/AAqAvhDRR/04w/8AoArYrK8Nrt8LaOD2soR/44K1aBiUtJS0AFFJ3ooAKWkooAKWkpaAEoqlpWs6brlq91pd7DdwJK0LSQtuAdTgj+o9QQRkEGrtVKMoNxkrNABrzv4RYOka24H3tYuD+orv7ieK1tpbieRIoYkLvI7BVVQMkknoAO9eefBlxN4Vv7lWyk+p3DocYyC2RRyy5ea2hL3R6RRWbr2uWXhvQ7rV9QdxbWyhm8tdzMSQAoHqSQOcDnkgc1zlj8StLTwpYa54iifQxfMwggmzK0qjkOoUbipGOSo6jsVLb0sHXqw9pTi2r206u17JbvTtsNySdmdtSVj+HvFeh+KoJptF1BLpIGCSgKyMhIyMqwBwecHGDg+hpniLxhoPhP7N/bd/9l+07vJ/cu+7bjd91Tj7w6+tSsNWdX2PI+ftZ377b7BzK1zbpa5v/hPfC/8Awjn/AAkH9sQ/2Z5vk+btbd5n9zZjdu74xnHPTmqlv8RdD1fTdSm8OSPrN7ZQGb7DCjRyyDp8ocAkZ67QSMjgkgG1gcS037N2Ts3ZpJ+bei+YuaPc66lrnvBvi2y8Z+H49Vs0eIhjFPC/JikABK56MMEEEdQR0OQOgrGrSnRm6dRWa3Q001dBRRRWYwooooA83uAW/aBtOOE0Jj/5FNekV53Hh/2gZP8Apn4e/L98P8a9EoJiFFFFBQUtJS0AJRRRQAUUUUAFGaMUUAFed/Gc48Dxr/ev7cf+PivRK84+M43eELJfXU7cf+PUCex6DbD/AEWL/cH8qmqOEYhQeiipKAWwUUUUDCiiigAooooAKKWkoAK57xr4mXwl4VvdVMTyyRrthURF18xuE34xhc4ySR6DkgHoe1ZXiezn1HwnrNlax+ZcXFjPDEmQNztGwAyeByR1rfDcntoe0V43V+mlxO9tDzaw+Ken6l8K7qXXroxao0M1mcQMBcy7DtKYyDwV3dApYZChly/wF8RPDeh/C6z+2Xcgm05BBNCkLsxkbzGRQcbTuEbYOcDuRXA6p4e8R3/wx0fzvD19bR+H5rhJxMpSSWOVlfeqEbsLyGOMcgjPzbc3QfB2oXvg++1Y+FbvUIXlt1t5obhkmVQcytFGFPmKwwuSDtzkbtrY+xnlGWTcpuVnzbKUbL3rJa23WvktN1Z83PNHq+rfGPTb/wAD6vf+Hnmg1S32JHDdQZZQ7Kvm4Usu0ZPJOA20EfMobtPBXiVfFvhSy1YRPFLIuyZTEUXzF4fZnOVznBBPoeQQPC/DvgXxDqNn4otLLw/e6fb3FjGIF1RQJGkWaNwgkKITkJJ0AXO3d0Br2P4aalqV74TtrTUtBvNKfToorRDcjHnhEUbwCAw6emORgnnHnZtgsHQw8lh7NqS+0m0nFaeet9r2Lpyk3qY3xh1O9/s3R/DOm3D293r14LYydEMfCsrMMsAWkTOByAwPHBx9Qv8AxRF4utfh/wCBL77LDpFipnuL7bIW4U5LMGO0BkACqMFiMbQMXvjJ/wAS6/8AB/iOb5rPTdTHnInMjZKP8oPB4hbqRyR+FTXo9f8ADPxKl8baFo7+INM1WzjjYWvzEZVcbSm44/dI2/btw2OuDWuBjD6rSVotuM2lK1nO6SvfS/LtcJfE/l9x0Hwt8Watr1rq2meIPm1jSbnyZ3CIoYEsADtOCwZHHAAwF6nJrK8eyfEXQ/7V1y18TaZbaHBhoofswMgBwoXBjfLFiBktjJz8o4HP6EfG/hfw/rHiq20F5dX1zVVL6e9lKxjjAlZpNitvUF2wN3QAHncDXT/EPQte8b6z4d0RLCa20M/6ZfTtImUYcFCQGw6qxAwSGL9whITo0aWY865PZPe9mlypOVk/O6Vgu3C2tyOTxL410/4MRa68SXurzr5pmWJQba3bJWUqvyuQuDwBgMCwO1s27G1uvih8GYBqM+zULqJyskbmJGljdlQuBkFSVBYYI5yACFx1viHTGuPBmq6VptugaTT5ra2gjwigmMqqjoAOg7AVzngmRvBXwgs7jXYXtDZQSzyxOQHw0jsq4JA3EMoCkg5IBwa4liIToe1oRUavtU1bezTsrdk7LsVZ3s9rEnwl8RT+I/AVvNeTTT3lrK9rPNNjLkYZTkdfkZASeSQc56nuK8y+C2mT/wBgah4mvbjzrzXblpnIwBhGcZIAGGLmQ8cY24xzXpuK4s2hThjqsae1/ufVfJ3RVNtxVwpDS0hrzizzb4MkNoGuMAQDrdycf9816UK82+C53eGdXbOd2s3J/wDQa9JpLYmOwUd6KM4plBSUtFABRSYpaACjNFFABRRRQAVwHgjDePPHLA/8vsI/8hV39cB4EU/8Jt46cjrfxD/yHS6iZ39FGKKYHmtiD/wve/3A8aYmM/WvSq83sSf+F6X4Jz/xK48f99GvSKS6k09goopaZYUlFFAC0UlLQAUUlFABS0lLQAlFLTaAPOLNcfHm/Of+YTGf/HjXpArzawz/AML41LBODpUe4f8AAjXpNJEx2DvRQaKZQUUUtABRSUUALRRSUAFFLRQAUlLRQB5xoRP/AAu/xOO32CA/yr0avO9E/wCS3eJf+wfb16JSRMQopaKZQlFLSUALRRRQAUUUUAFFJS0AFIaWkNAHm3gkkfE/x0Mf8t4j/wCOCvSa818DNu+J/jrk5+0Rf+gCvSqRMdhaKKKZQUUUUAFFFFABSUUUAFFM8weZswc4z0p9ABUczeXC7eik1JUU4327jOMqRmgT2PPfgfx8MLH/AK7S/wDoVej15x8Dx/xbCxPrLL/6FXo9CBbC0lLRQMKQgkHBwaWigBB05paSloAKSlpKACiiigArzj4sf67wh6/27b/+hCvR685+KYBvfBn/AGHrf/0MUCex6KDS0CigYUtJRQAtFFFABSUUUALRRRQAUlFLQA09DXm3wf4svEg9NauP/Qq9JPQmvOfhB8+meIJ+0mtXB/8AHqBdT0iiikoGLSUUUAFLRRQAlLRRQAlLSYooAKO1FFAHnOsAH48eGwe2l3BH5mvRq851M7vj1oQ/uaTP/OvRh0oEgpaSgUDFooooASlpKWgApKWkoAPrRR3ooAK4T4xN/wAWr1kevkD85467uuC+Mxx8LtU95Lcf+R46BPY6/RF8vQdOT+7bRD/x0Vfqnpv/ACCbLP8AzwT+Qq5QMKSlooAKKSigBaSiloAKoazYz6no13ZWt/Np888RRLqAAvET3Gf6YPoQcEXq53xZ400rwbYC71Pz23MFjjhTc0hPpkgdATyR09cCtaEKk6sY0leV9Ouona2p4H4Z1rXPCXwzvtb0nVXiN1qqWIt2jV0jIj8xpRuyNxAVemMZzk7StrRvFPxM0qHVdPZtTM8di19/xMQPMt41dN0o84Esu1WXaOMsSBkUW2tfCq2tdUtRpniZ4L/BEbmIi3IJKtH8/wB5dxALbjjI6MwavY6h8KLO1vYH03xLdNdReWJbgQF4Oc7o9rABsgckHpjoWB/R5xjNzlPDuTbT1gnfa3Vba77nGtLai6RrfjGA61oeu6jqcCXmkXMhh1NZGkcJE7Dy/MB252sCeAV3YO4KR6V8C7SSDwM9y91JIlxcuVhYDbFt4OO/OMnnHTAHJPG+Al+HD+J1j06DXpr2S3mjhj1JYmibKEOCE/2C/wB75cZ74rpvgxpOn6Z4av8AXzLOslxLJC6GU+WEjdgML3Puckc4xk58PPcVRVOeH5XCT5ZfCle11306a67NGlNO6Zc+PNxLH4BtkjldEl1CNJFViA67JGwfUZVTj1APas7xfZ6bcfG/wlo+oRw/2PHYjy7SQ7YFfMoRQvA5ZI1x/FhVwRxXb+L9Ch8d+CLixtZYFlmCy200ybgjqQR7rkZUkcgMeD0OBp/hCXx54KsrXxzptzaanpzPbQ3CXB811UqDJyWBLbMEtuzgsuAwrjwGLo08LBylblc4u2650rSS0va3TVFyi3Iw/CtxpHh342eLILW7trDRY7MPIonCQJJuhBzk7QQ7uoH8JYqMdKo/EexuvEfxd0C20WbT3mutKD28t0izQMuZmyQVdWBUHBwecH3ruLH4SeHdP8MapoUM2oeTqbRtcTtKplxGwZVHy7QAc/w5+Y89MS6v8KPDetaNpmnXBvVOnRCGG7SYGdoxn5GZgQVycgYwvRdoyK2hmeDhiVXUm3y8l2r3XKlzNX113V9uouSXLY8KluopPEun+G9atdPt47bWjHqk9ri3huVDrHllUKqhFEmGAXh2OASxb0p7PTdF/aK0i00OOGzinsW+2W9odqb/AC5TtZBwOFibGB2bGTmurg+EvhSHwvJoJtZpIpJfOa5aXE5kCsqsWAAO0OcKRt7kEkk0LTwFafDfStW1rwvaXuq6wbby4YbmUH5dwLYCqu7oGx1OwBSCeeivm2FxCcKTabjKCW0W5W9562SXZ7K21hKnJbmb8NZl0/4keNNC08PNpKzmdXjQxw20gYgxBMYB+YrkYyIcgEdPWK4v4Z+Er3wt4embVnSXV9QnN1dSfecEgYRpOrkHcSemXbGep7Svn82q06uKk6bulZX7tJJv52NaaajqFFFFeaWFBpaQ0AedWK7/AI+6pID/AKvQ40P4yg/0r0QV51pGX+O3iNu0el264+pBr0UUEx6i0UtJQUFFFFAB3paTvRQAUUUUALSUUUAFec/GAeZoGkxDrLq1uoHrzn+lejV5v8XGAtPDaEAh9ahGCOvDGgT2PR1GFAFLSCloGFLSUUAFFFFABS0lFABRRRQAV5X8XtS1SDUfCul6frNxpUOo3TxzzwOUIw0ahiQQSBvY4yAe/QY9UrzD4u+ENb8T/wBh3GjWUN6bGWTzbeSQJuDbD/EVBX5CDgg8jHcj08nlTjjYOo0lrva1+V2vfTexFS/LoeVeKNW1DQpo4LL4gXmvRSiWOePzWZAmAvILsDuBfHptz6Y92+F//JM/D+Bj/Q1rwi/+G3iez08XFz4asdMtLNZJpriO5Viy4Bw37xyfu4GB/Ec8cj3r4aqV+G/h4H/nxiP6V0ZxNSjR5pRlOz5nG1vidvh02Ip/Ezq6KM0V4hsVdT02y1jTJ9P1C3S4tJ12SRP0I/mCDggjkEAjmoNB0Ky8N6Ha6Rp6uLa2UqvmNuZiSSWJ9SSTxgc8ADitGitPaz5PZ39297dL9xWV7h0qOGeK4QvDKkihmQsjAgMpKsOO4III7EEVV1mLUp9Gu4tHuYbbUWiIt5p03oj9iR/XnHXDYwfnnwV4r1zwT8OtQ1e0+xXFnPqa2sNvOjEpN5e95CQRldiqu3PXnjBD+jgcrljKM505LmTiku9/6/BkynyuzPpSsbxL4X0vxbpsdhq0TyQRzpOoSQody9sjsQWU+zHGDgjw/wAP/Gbxj9i1GOW3TVp4oDcRy/Y8+UAybjJ5ZUCMJvOcZ3EZOKg0T4leKvEGn6/o+pXltdRXGlXLiSaOONogkTM20Lt3lhkY5I4borA+jDhzH0JuopqPI1qm7+q06edr9CPbReh9E2X2T7Bb/YPJ+x+UvkeRjy/LwNu3HG3GMY4xUep6nZaPps+oahcJb2kC75JX6AfzJJwABySQBzXCfBOLUk+Hlu93cwyWckshsokTDxIHYMGbvlwxAxx6nICwfHa8ntvh9HDDJtjur6OGYYB3IFd8c9PmRTx6V50cvUsy+p811zWv89fn+pfP7nMdVo/jjQ9X8OQ681z/AGdZTStCraiVgy4zwCTtbofuk9COoIGvYapp+rQNPpt9bXkKtsMltMsihsA4ypIzgjj3rybxjodlq3xZ8H+D7hXGh2+nlo7dGwQFEny7/vYIhjB5zgHBBOal8B6fF4Z+M/ifw7pjOmmfY0nETkMQ37tlG4jOF81wOehGckZrpq5Zh3RdSnJqXLzpPbl5rWv3+X+ZKm72foTfCLWtK0nwbdNqep2dkJ9VuTH9pnWPfjbnG4jOMj8xXpn9taV/ZX9q/wBp2X9nf8/fnr5X3tv384+9x168V8n6Dplxr+o2VtpemDVr5BOZrOQMkIQOxDGRXUj73qoztGTuwPVfhnoHh7U9G13QNcTN1/ae2fSpHKxW0q79ogYMSzFUkBYNuKpg5A3NUspoQwcMTObvo2klezdtr39G9H31JjN3sek3Pjbw7Dpt7e2+q21+LOBriWGwlWeXYMZO1STjJHJwBnJIHNW/D3iLTfFOjQ6ppc3mQScMrcPE46o47MM/yIyCCfFfhrok/gn4rLouv6bC17dW0hsrlGEm3G751O75VZUccru6DgFs9P8ADCaLQvHXi3wdBKj2kU5u7RYGDxxLkKylz8xYBolIOcFG5z1rG5Vh6UKioycnFRknpZxbs9uz/Xtq41G2rnrFFFFfOmwUUGigAooooAKKM0UAH8Nef+AQP+Ey8dN66jH/AOi67+uB8And4s8cN/1E0X8kpdRPc9AooopjPNrBmPx01HngaXHx+Jr0ivN9IJf4461k/d06ID6Zr0gUkRDYKKWimWFJS0UAJRRRQAtFJS0AJR3paSgAooooA8207LfHnVzjhdLiH616TXnGkYPx017J5Gmw4/OvR6SJiIelME8TTvAJUMyKrtGGG5VYkAkdQCVbB74PpUleAWs/iTRvjN4n1Ga8sri40+xlu70LEVS4tlRGWNByUbHlDOTjBJL4Ib0cBgPriqWkk4xuvPVL+vOwpy5bHv8ARXzlpHxs8VzeKLd7mOG5s7iWOJrC2tckAsoPlc7i5wcBmIy3TpiOH4x+NE8WR/bPsyRrOIptMeNYIwfuspd/mQ5ycs2AevAxXqPhbHJtXjor7/htv+HmR7eJ9HRzxSvKkcqO8TbJFVgSjYDYPocMpx6EHvUleMfCyHV/+Fm+NH+2W32SO8kW+QQkGaQySbGQZJQAh+rNwcYJ+ZfUvE95Pp3hPWb61k8u5trGeaJ8A7XWNiDg8HkDrXl4zA/V8SsPGXNfl19Ut/v+4uMrq5m6N4+0DXdS1a0sbh2i0tQ894yYtivOSJOmBg8nGcErkAmtXT/EOi6tO0Gm6xp95Mq72jtrlJGC5AzhSTjJHPvXgd//AMSz9nHS/sf7v+1NTb7Z383DSY69P9TH0x933Od3X/Cmm/D/AOIPgSbw/wCdDJdXItpzI/meYNyIzcjhmWVgcYHTAFevUybDOUoQk025qK3u6a1bfS72tchVJf15nsuoapp+kwLPqV9bWcLNsElzMsalsE4yxAzgHj2qG08Q6LfwXM9nrGn3ENqu+4khuUdYlwTliDhRgHk+hrlfix4avfFfhqx0zT5bZLo6hG6rcS7N42ODt9SAS5A52o2MkYPDeC/Ddr4V8Vz+BvE+l6ffza5Z+Yl1bszbUG4+WxYKQMxFgVAIYL14KcWGy/D1cI6zm+dXfKrfCt3rbpcpzala2h65B4u8NXM8cEHiHSZZpWCRxx3sbM7E4AADZJJ7VV8OeONG8UX+oWFi80d5YysktvcxmKQqDjeFPO3PHOCDjIGRnyZfCfhnUvjPZ6Boeloum6Wpn1FhMZRI687TvdgVDGNCoAOS4PTI6PxFPF4X+O2h6lDKgXW4BaXcMbB5WYnYjMrfdUkRcgjPlvx1z0TyzC/w6bk5Sg5q9la2tmlfdJ+mnfSeeW77mnoYP/C7vEn/AGD7f8a9FrzvQwf+F2+JTj/mHwfzr0SvnEaRFoooplBRWV/wkujf8JJ/wj39ow/2t5Xm/Zsndt64z03Y525zjnGOa1audOcLcytfVencL3CiikqAFoorKsfEujanrN9pFlqMM2oWP/HxApOU7HB6Ng8HGdp4ODVxpzkm4q6W/l6hc1aKKSoAKQ06mmgDznwThvij45Yf894R/wCQxXo/avN/A/HxM8dADA+0xHn/AHBXpFBMdgpaKSgoWiikoAWiiigBKMUUUAFFFFABVe+yLG4I6+U2PyqxUF24js5nPRUJP5UCexwXwRIPwt07HZ5c/wDfZr0TtXnfwRXb8LtOPq8p/wDHzXolALYWikooGLSUtJQAUUUUAFFFFAC0UlLQAlecfFAltb8Dx+utxH8iK9Hrzf4n/Lrvgd1++NaiAHsSoNAnsejiloFLQMKSlooAKKKKACkpaKACkoooAKWikoARvuH6V518GcHwlqDf3tWuv/QhXoj/AOrb6V538FOfAksv/PXUJ3/MigXU9GpaSloGJS0UUAFJS0UAFFFJQAtFFFABSUtIaAPOL1l/4X7pobr/AGPLj67hXo46V5rON/7QVpkA7NFkI9vmH+NelUCQtFFJQMWkopaACkoooAKWiigBKWiigBK87+Nj4+HE6f8APS7t1/8AIgP9K9Erzn42f8iCo9b+3H/j1Amd/ZrssoE/uxqP0qxSAYUAdqWgYUlFFABRS0UAJRS0lABXlPx9Zf8AhB7EDGf7TT/0XLmvVT0968f+O8co8JWbyHg6ggH/AH7k7V6uR/8AIxo+pnV+BnMy+LPHVncJp/hj7N/YYj/0IzRqcoFyRlupHtxXPQ6z8RdIvYCttNBEfmIgVAJTIeSXIOSST9M8Y4rQ+INlqdtr+lIrSEPOyooGAucAAD0wK6678NLpmkSzO88zoQ0EMjZVGOMBfXn1/CvINkc5c2GtS/E/SIr3Zpl9Pp0sgaJi7quybO9iSWc4IJ9MV1nwg8I6dN4NttQvIzeySzPiOf5okAY8hT9O9UNfSaP4zaI04IkbRpmxnp+6uP8ACu1+Dwx8MNH91Y/+PGvWzT4MP/17X/pUjGO79Tsrezt7PctvCqK3UL0/KrIpFBFLXlmgtJRiigAopaKACikzQKACud8V65NpVvFDakpcSnO8x5AUdcE8Z6evHpxXRGsDxdY3OoaTFFawmVxcKSox0wRn8yK48f7T6tP2T963Tc4Mz9r9Un7FtSt03+Rm6d4rmS8ZdRfdbrbRsXSBgQx25J9vn69DgY64PTtfwLqUenneZ3jMvCEgKDjk9s8/l7jPOX+mb9d1m4vh5NhLaACdugb5McA5JBXp9PUZf4NspGgk1S4OZJVEMR9I1AHb/dA5Gfl964cNWxMKvsJa6vV72Td/v0seZg8RjIVlhpe9dvV7qKbu+9noov1Ob02/Sx+LHje9kXcsFlaAe5wcD8TgVqmS90jQG1lp5G1DUXUbiRhF5IO3kHIH4A4GMHOLYWUuqePPiHDbgGYpYKoJxnAc4/8AHa351l17wRarZx7pbRlWSMZydikcccnBBx+HJqswc3Uaje6i3H12fzS+648zdR1Wo3uoNxt/Nezt5pbdVe6LVlqOraf4jg07V7uGZbiPKlMKFJzjnaMnKkY962tWh1SaCMaXcwwSBsuZFzkY7HB/l+I788q6lreuQ382lzQw2UZZYJnKh5BkrtJA5J257cc9hWl9t1i78LXMzWRhvyGVEUEErnlgM5BxnA65Ge+KWHq3pzg3JrVxet7K3X12Hha16VSnJzcdXF+9zWSXXffYxIda19bLUrpr2GWG1xEH8oFWYsBlCAM4HPOeo454tWuq63ZXmltf3ENzb6jgIiqAVB28nCjkbh69/rWjZ6M1l4UkshbRz3EiF3ikbCs57Zz2wBwRyOo61zGi6Jdy63ZsbK6to4SskjzLwSpzxkDqcDHJHXmuOccVRlTV5Nu3V6O+t+j00123PPnHG0JUVzScpJdXo+bW/R6aavTc6Gwln0nxNJpMsxmtroNPBnJMZJJIJJz2b1ycHjJrpa5dXGp+PFmtgTHYRGOZmUgbvmGB+Ld8dDXU16+AfuzS+FSaXp/w9z3ssfuVIp+6pNR9NPwTuhO9Bo60YruPSClpKKACvN/iviSfwlCed+tRnGPRWr0ivN/iaN+v+CI/XVgf/HaCZbHo4pe9AooKDvRR3ooAKKKM0AFFHajNABRRRQAtJS0lAHMfEJmT4fa4VIz9kbFO+H42/D3w+AB/x4Q9P90VB8SWK/DjXSP+fVv6Va8CYHgDQMdtOg/9Fign7R0VFFFBQYoBoooAzdc1/S/DemnUNXvEtbUME3sCSzHoAoBJPU4A6AnoDXglvZ/DqHRtU0mXx5eTWNxKJ7OI2EwFtKMgSH5fnbadpxtBGeM7Svb/AB9P/FDWP/YST/0XLXk/iCa18OaqYre2s5rJWYxn7HG0uewYSKQRn0r6DB16WAwsaspTvUb+Hl+xa26ffoZOLnKy6HR6SnhS/wDtn9sfErUbjUr62+wwzslxGIVL5w7NwyHjKsQoBbPOGXvtI+ELw6+NU8QeJr3XNttLbCOdWUlJFZCC5djt2u/Axyc59fGtTvrrVPAjXF3oGnWRj1KNI7y3s44JJA0cjFDsAyANvb0r6xrfH5jVWHhWw85JVOZNNRurWWjUVa9+hMYK7TWxx/gjwNP4LkvIl8QXt9p0nFtZTKAluNxbPU/NzyV2g8kg8Yf8SvC8vi3wVdWFpEkl9Gyz2oeQoN6nkZ6ZKF1GeMsM46jrqK8T6/XeJWKbvNNO9rbd7W+fc15Vy8p5PB4db4q+GdM1a+OoaH4j0xjam7MIUvIjLufACsQGDYAK7HLjnHM1r8G4oPDuu2M+tvdalq7RmTUJbYFkVZBIRgsWJZhlju5+Xjjn1KkY7VJ9BXS84xMfcovlhe6WjtrdK7V7J9NvIn2cep8+fDr4eXHiHwra63pXiG70O9Dz28z2yn96gkyOVZT165JBwvTHPZj4LWS6G8Y1m5/t97xbw6yUzJvBOABuyB8xJIbJbDEnAAsfA0f8Wytv+vqf/wBDNek0lnOOSSU9vJfjpqvJ6eQKnHseVx+DX8BfbfG2s6rqfii/062ItUYMGjByGJJdjtAY5PRQXOCcY1fhR4d1LSdGv9V1yHy9Y1m5N1Pu4fYeVDqMBW3NI2AONwBwRgd/RSrZpWrUZU6mrla720W0UlZJX182NQSd0GMc0UUV5hYc0UUUAAooooAKKSlFACGuC+Hx3eIvGr9zqxX8lrvj0rgfh2uNZ8Zc5zrMn8qXUl7o76iiimUea6Pg/HLW8A5/s6LP516VXmuisB8cteX1sIq9KpImGwUUd6KZQUtJRQAUtJRQAtFFFACUUUUALSUtJQB5zpRA+OuuA9TpkOPzr0avONNOfjvrHtpcX869HpImIyeeK2gknnlSKGJS8kkjBVRQMkkngADvXiV5f+AdZ+Ib67H42mgi1CIWt5ZG0lRJ0KeWUMpUBEIC5yOMEhlOCvqnjX/kRPEP/YMuf/RTV8qXGt28/hS10YaTZR3EE3mfb40AmkGXyrnGT99e5GEH4fU8P4P2kZVE5Jt8nu20TTbbunpou3qZVZW0Pc7D4MPaX9mk3i3U59Fs7n7RBpw3R7CCSuHD4VsnllUE5ONpORBdfBO7vpBBd+NtTuNKFy04tJkLnliSdxfbvO5svt6sTjnFet0V5v8AbmP5ubn19I/ftv57l+yj2OIg+HP9n+PZPEmla7e2Ntcy+fe6fGNyXEh3ZyScbSWJwVJGW2lcjb2N7ZwajYXFjdR+ZbXMTQypkjcjAgjI5HBPSpqK4a2KrVnGVSV3FJJ9dNtevq9S1FLY8Z8IeHbrUNH1T4ZeLLC5RbFhd21/AqlFRnyNjleCx8wgnJIMinbtxWz4a+EP9j+JLDV9V8QTax/Z8QjtYJoMLHjhMFnbCrkkAYwcEHjn02iu+tnOJm5+zfKp7pd2rNq+qv1sQqa6nldr8FktvC50seIZheRXy3tpex2qobd9oU453c7QThxyiEAYO7V8LfDJ9F8SLr+s+Ib3XdQhiMVrJcbl8kHcG6uxbhiAMgDJOCSCO/pazqZxjakZQlPSV76Lrvra6v1S/UapxXQ5jwd4JsvByag8N1c3l3fzmW4url9zuMsVB7EgMct1YkngYA8cHiXX9f8Ajlpup2ekvHMGaCztNQ/c4gUSJIWIGQQfOJ+8VYFfm24P0VXkvjOC3uPiPpXiLSvGXh2yutOT7Ncw3lyhZAGfcNufmJDupUlSMcEE5HdlOL9pWrSrrmlOLV3ey02suj0XktFuRUjZKxwifFxrL4iah4ks9KElrdxC3aCaXa5Rc7WDAEKc4JGG7jPetzVvj9fRa6yaVpdlLpcUpXdKz+ZOgY/Mp42blxgFTg9c9K47/hFNNfxhqeh2HijRo9JHlsL+9eM5jLA4jbGC69DtK7sc4BIHR+J/Ds2s6rqUiePfBt3bXcquLi8mt0ucBVABdIyVwFA+UgHBOBuIr34YTJ+eNqatbrz+W+m+/X/gYqU7bnQ6FrviK9+PF8ILZ1tZ7OI3FpdTsv2a38uNlO3HEgL/AHMHDSOM4JevZq8uX4a6/onifTdY8M67bROLO3sr/wC1wZDpEsaEooB4YRgldykEcPzx6hXy2bVKFSVOVBqyilpe+mmt/wAPLc6Kaavc+ffDeoS2/wANfHHjmFUj1u9vGgMiAgQrIyFjGQdynMxP3jyienObqPhT/hAvCfhXxzpmozPqMssMkkTjEZ8yMyBRtIO3aCjDJ3Bj93pXSeGtLgsrrxN8KdXimtotQlkuNKnkQsZABlXLKQDgRIwHAyrqSD8tW4/hP4svZ9K0rXfENte+GNOn3R24ZxI8YPCkADkj5RlzsDHaex+neMpUasueajFvms18VPksku+t1bQx5W1ov+HPTfFPiSy8KeHrrVr10AiUiKJm2maTB2xjgnJI9DgZJ4Brxn4T+JJ7j4oard6zqUMUmq23meWboGOSVnjMaLljllViqrksoyvGCK7+y8B6jqGqeIY/Ft3DquiX1z59laPNK72+HYrtYkeVhW2kLnPTIAw1Gw+C+g2njK41KSCGbR/KjNrp7l28uUEbixLHcvy5wcg7yCAFGfGwlXL8Nh61CpJuUlulddGktd779NNzSSm2mjH+z6vpv7SVkL3VHuY76CWSIKSoW3KSlYivTCsme+SAx5Jxe+I8EXhb4geGPG8cSRwmf7HqErKCoUqVDbV+Zm8syc8/6tRjsep1DwbLe/E7SfFgvEWGxs3ga3KEszHeAQc4xiVifTaOu75eO1uSH4i/F3TtKitHuNG8OtIb6UxgL52eUbdkMpaNFxjJ/eYyORpQxEa1anVv7kaTU7K38yt0V3pbz7iasmvPQ9fpaSlr5Y3EoPalpDQB5z4JJHxM8dRkH/j4hbP/AGzFejV5t4Kfd8UvHI7edD/6ABXpNImOwUUUUyhaSlpM0AFFFFABRQKDQAUUYoxQAVXvEEtnOh6NGwP5VYqpqLFdOuWXkiFiB+FAnscL8EM/8Ku0/J/5aS4/77NejV538FBj4WaXyDlpenb94a9EoBCUUGkoGLRR9aKAClpKM0ALRSUUAFLSUUAFec/Eog+KfAaHodWz+QFejV5x8ShnxX4D/wCwt/QUCex6OKWkHeigYUtFFABRRSUAFFFHagAoo5ooAM0tJRQAyT7jfSvPPgmwb4cxAD7tzMP1r0OT7jfSvPfgoP8Ai3kbf37qZh+dAup6NRSUtAwooooASlpKWgAooooATNLSUtABSGlpDQB5yuD+0B9NCf8A9GR16NXnER3ftATY/g0Mg/jJHXo+KBIKKDRzQMKKAKKAFpKWigBKKKWgApKKKACvNPjcvmeD9OQHltWtwP8Ax6vS681+M3zaJ4ej/v69bD/x2SgUtj0oUUCigYtJS0lABRS0negAooooAK5jx34Ni8ceH10yS8ezeOdZ45VQOAwBXBXIyMM3cc4PbB6elrWjWnQqKrTdpLVCaTVmeQSfB3X5XjeX4h6k7RkFC0Tkqfb99xTpPg/4hnKNL8RdTcxtuQvFIdp9RmbivXKK9D+2sb/Mv/AIf/Ik+zieTx/DG60W8ufEmreKrzWLi0sZ0hE8ZBG5GXlmdjtAZuBjk5z1B6L4TRmP4ZaJg53QZ/U1veK22+EtXPpZy/8AoJrK+GKbPhroA/6dFNceKxdbFTU6zu0rbJaeisgjFReh1o6UUUGuYs4Dxp8ULDwl4k0rSv3M/mSg6i25t1rEcYOAD83O7HXC9PnBG3qPj/wrpV1a211rtkstztMYR94AYKVZiuQikMpBYgEHOcVwPxsjtbLXvCGs3mn+fZw3LLeMIQ3mRho2EbE8HIEmFJx973ry7xlp0Vv4v1+XVv7QspbmeS8sU+xgidJGZlLbnUoOgPDEHcCAVIr6/AZNg8ZQoyd4txle2t2pW7dPTa3qc8qkotn0Zq/xE8JaG8SX2u2waVQ6rDumO0gMCfLDYBDAgnGQcjNY+r/FHTdJ8e6ZojzWTaZdWwllvxPuETvkx5xkBSADk9pFbIA+bwfxHpNjps0EWpHX7PUP7Mt38q9tkk8yXYRgNvUpEAEUcMwwwIBXFdHZSf8ACNXPgLxTrGiTDR4LF48Rxbsy+ZOyNh24Y70kBJAPJXgYG6yDB06cZpubkpK2iu+Vtcv3ea79he1k2fSleVjxBqWt/FLVrhdams/DHhaJmufs6cSuF+dZFOS3KychTgR/LgsGPqEEy3EEcyBwsihwJEKMARnlWAIPsQCK8d8M6fLJ4r+KXhqRkh1LU1kkt0kJKlH83DFlBAGJ4zjr83Tg48HK4Q5K05LVRS72TklJ28k3r0NZvYq/8Lb8c/2V/wAJJ/wjFl/wjv2ny/Mw+7buxjdu/wCA+Zs27uMZ+Wuv1LWX1C5v9Qt9VuotMttOF/GbcEF4hGr8KSvJDZ5+n08pm8XS2/wvHw7m0PUI9bM6xhXQglWlEy/IRu3EkKFxyCDntXW2FxcNq+teCIrYT3sfhoWkc0Dlkll+zRDGSoCqSSAzEDoOpArqz3JlXVNU6SilNt2la9JW95692ttfI8zGUp11CCu1zK+ttLP062OZ0Hxp4r8R3cNuwju7aSZIZLeK6AnYEjlI3lBYDOc42gA5KgEib/hLfGM1tq194bgluPD+mysv2lfMUFM/e27genzEAfKD83rXLJHpsmj6ZpOlaTqNv41gvT9ouCxjChS5wMv8hX5CSVXbsJJGDW7pfitvAvgvxJ4O1PSrj7deGUQyggRssiCMtkjJUBdykZDZ7da9Wtw7lyrOpSw8XPRKLbXu82src2vk9Ot0Qsvw3NzuOtrXu/uK1t4r1BfE48QWuoT2mmXElrbalMHJwWUnkDDOVAkweT8p5wwFe423g26td32bXJod2N3lxlc46Zw1fMWna7bweEdd0wpDJLdXNq0ZaMsUVBKXZT/C2Si+pDMO9fRnwrv55vDaW+paxZ3upNiZ44rgSyxqRx5hycsepr5jOcrwUqVKaj8LnGNm7uCejut+qu9XbyZr/ZmGqNc8fhWmr0/E3/B15cXmjO1zM8rJOyKznJxgHr35Jroa5fwL/wAgSb/r5b/0Fa6evCy6TlhYNvoa5TJywVNyd3YKKDRiu09Ap6bpNnpMTx2kW0OxZiTkn0GfQdB/jmrtFJUwhGEVGCskRTpwpxUIKyXRC0lFFUWGKKO9FABXnPxBw3jfwHFzk6hI2PYKP8a9FrzzxoQ3xN8Bx4/5aXTfkqf40Ey2PRBRRR3oKCijFFABSY9KWigAooooAKKM0UAFFGAaKAOP+KTbfhjrx/6dv6itXwigi8HaNGDnbZQjP/ARWJ8WW2/C/XfeAD9RXReHE8vw3piYxi0iH/jooJ6mpRRRQUFFJQCM47/SgDyv4+5/4QWyz/0E4/8A0VLXlnii50HWtdvbyHWbfyXlUxjyJlyvccJwPfqTX1DeWVpqNq9re20NzbyY3wzxh0bByMg8HkA/hWV/whXhU/8AMs6P/wCAMX/xNepTxODqYaFDExl7jbXK0t7d0+xFpRk3E+d/EWq6H/wriw0bTtUS6u0vvPkhWGVQi7XGdzqM9VHX0r6kAxWPD4R8NWs8c8Hh7SYpomDxyJZRqyMDkEELkEHvWxU43FUKlGnQw8WlDmerTetuyXYIxabbCiiivNLCo5ziCQ+impKq6icabdnpiFjn8DQBwnwRGPhdp59Zpz/5FavRa8/+C4x8KNHOBy05/wDI8legUCWwUUtJQMKMUUUAGaKKKAAUd6SloAKM+1MzliOeOacM0AL2rgfhp8114ukIxnXbgfkcV31cH8Mh8nip+58Q3g/JqBPc72imbh7/AJUUDPN9I2/8Lz1sjqNOiz+delZrxa813UNC+NOtS2Gh3Wqu9nErRwHBUYBzzXRH4ka+v3vh7rX4MppIiLsj0fNFebj4k68TgfD3W/xI/wAKB8SfEDHA+HutfiQP6UXQ+dHpGaM15wfiN4hAz/wr3WP++lo/4WN4iz/yT7V/++1ouHMj0eivOR8RvEH8Xw+1n8GWl/4WPr3/AET3W/8AvpaY7notFedf8LH17/onmt/99LR/wsfX/wDonmtf99pQFz0WivOh8RPEB6fDzWv+/q0f8LF8Q5x/wr3WP++1oC6PRaM153/wsLxFnA+Hur/9/Upp+IfiXB/4t7q3/f1aBcyE0vB+Ous47aXFn869HBrwLTfGGsx/FLU9TXwjqD3MtnHG9kP9YgHRifSu3/4WPr3/AET7Wv8AvpaSFF6Ho1Y0PhLw1bTxzweHdJimiYPHJHZRqyMDkEEDIIPeuT/4WPrwPPw91vH+8tH/AAsnWeP+Lf67k/StIVJwuotq49D0WivO/wDhZOrquZPAOvr9FBoHxN1Aj/kRfEOf+uH/ANaoDmR6JRXnY+Jmon/mRPEP/fmj/hZepH/mRPEP/fmi4cyPRKK88PxK1TPHgPX/APv2KQ/E2/GQfAviLI6/uM0BzI9EFFee/wDCz7kAFvBPiQeuLQmm/wDC05QefBfib/wBb/Cgd0eiZr57+Gng3w7rvge+1LVdLe7u4bx41ZJpFIQRxkDCsB1Y9u9egj4psevgzxOP+3Bq8Q8PyXyeF7gabP4miuhclv8AiWo727AKvDBT97+mK9nAVqlHAYidKTi7w1Ts/tdjObXMrnWaF4c8Gap8S9S0xrNBpsdqjW8LXEo+fjccht2fbNbHjnwB4W0j4faxqlhpIt722ljSJxcStt/eop4ZiDwT2rx+9OsXmpNJNPeyX0arjzoCJgfw5/Gt208VahB8Pda8P6na6lJcXlwspuJgxVCHjJ3E9/kx+NGW5ljJ4ylGVWTTlH7T7rzCUYcj0PpXwX/yInh7/sGW3/opa3c15H4Y+K+l2HhnSbCbSNbL21nDCXjsyysVQDIPcHFbX/C3dH3Y/sbxF/4Lm/xrzcV/Hn6v8ylJWO9METTpOYkMyKyLIVG5VYgkA9QCVXI74HpUlee/8Lf0IHB0zXlPvp7f40H4xeHwcGw1v/wBP+NY3Kuj0KivPh8ZPCwXMw1GD/rrZsKP+Fz+Dv8An6uv/AZqQcyPQqijgiieV44kRpW3yMqgF2wFyfU4VRn0AHauCHxo8GE8306/W3anD4zeCSedUkXHrbv/AIU7i5kd/RXBf8Ll8DZ/5C5/78P/AIUD4y+Bj/zGMfWF/wDCkO6O9oNcMPjB4Gb/AJjsY+sUn+FPPxb8C/8AQww/9+pP/iaA5kZvg3B+K3jkjH+tgHH/AFzWvSK8T8MfEHwtY/ELxXqNxqkcNnevCbeUo2HwgB7eoNdyPiv4G/6GK2/75f8AwoJi1Y7OiuPX4peCX6eIrTn13D+lSf8ACzfBf/QxWX/fR/woK5kdZQK5VfiT4Mfp4jsPxlxUn/Cw/B//AEMenf8Af8UBdHTUVzP/AAsPwf8A9DHp3/f8U5fH/hFuniTTfxuFFAXR0lFc/H448KSrlfEmk/jeRj+ZqT/hM/C//QyaP/4HRf40BdG5RWMPFvhxl3DX9LKjuLuP/GnjxPoJ6a1px/7ek/xoC6Naq96/l2M8n92Nj+lVP+Ei0U/8xfT/APwJT/Gqmpa/ox0y7A1awJ8l+BcKex96BNqxzfwTj2fC3S2/vNKf/IhH9K9CrzH4Natp8Hwz02Ca+to5Y2lBR5VBH7wnpn3r0Iatp/8Az/Wp/wC2y/40Ami5RVUahZkZF3AR/wBdBTxd27NtE8ZPoGFA7onopu9fUfnRvX1H50BdDqKbvX+8PzoEiHowP40BdDqWm5FG8UDHUlG4UZoAK85+I3/I4+AR/wBRRv8A0EV6LmvOfiCwPjjwEMjA1CQ8/wC7QJs9HpabkVQv9ZsdNurOC8m8uS8l8qDI+82M4/SgZo0lJvFG8UALRRkUmaAFzRRmjNABRRRmgAopKXNADZf9U30rz74Jf8kwsD6vJ/Ou+uWAtpSeyn+VcH8FsD4YaZ9ZP/QqBHoVFJmjPtQMWkozRmgBaKbmlzQAtFJmjNAC0UmaKACg9KKKAPN9OXd8fdYb+5pEQ/Mj/CvSa830rn486+RzjS4B+tej5oEhaSjNGaBi0lJmlz7UAFFGaM0ALSUZooAWim59qXNAAa82+MB/0Lwsvr4gt/8A0GSvSAeTXmvxbPmS+DYf7+vQfyP+NApbHpfNFGaM0DCikzRmgBTRSZozQAtFJkUuRQAtR+cnneVvHmY3be+KdmjjOcDNAC0UZooAwPG7+V4H1x/Syl/9BNQfD5NngDQhjGLRaT4iSCP4ea+xOMWMo/SrHgkbPBOjL6Wkf8qCepv0UZpCaCj558TfEnxnFr/iD7DrVva2un35tYrUWyMzAFwCNyNnAjLMSR1444HsHw81y98R+BdL1XUGRruZHWRkXaGKSMm7HQEhcnHGScADiue1n4LeGNa1m71OS51KCW7lM0iQzJsDnliNyE8nJ69+MDiu20DRLLw3odrpGnq4tbZSq+Y25mJJJYn1JJPGBzwAOK97MsVgauGjDDxSldfZSslGzTfW71MoRkpamlS0maK8E1CuW1fwFpuqeLtM8TRSzWWo2coaWS2O37SgBAV/0BPdcqexXqaM1rRr1KMnKm7Npr5PdCaT3I5oUuIHhkGUdSrDOODXCo8HhjX9Q+x2bGzsrWNPKjBJSIeUCQOScDn8K77Nee67cfZPE2oNIZo1nhVFaMckYXkZ7fKR+FeVmE4w9lOTslJfkzy80qRp+xnN2Smr/dIdrPxN8BS6dPZ3XiG38u5jaJxHG7MMjB4CnH41806p4m1GSN9Fk1L+0NKilATqA6qTt5OD09a9Z1bw5p17A628YSU5+ZlxuPqSMmuCuPhbfvITDe2wBP8AEW/wqv7Swn/PxF/2xgf+fiOINxGbN0ClHLDAUcY75/Su8+DOlajceP8AT9QhVo7S33tLITgMNpG0f3jnHFVYPhbqokzPdWRX0V35/wDHa9N+HmlWfhK6ku9QaSaYrtVYFBVRx6kela1c5oVeXnqp8qsvJISzbAL/AJeI9L8C/wDIEm/6+W/9BWunrlfBUscOiS+Y6pmdmG4gZG1Rn9DXRfbrUdbmHjr84rLLf90p+g8ossDSv2LFFUzq2nDOb6146/vl/wAab/bOmdtRtP8Av+v+Ndx6N0XqKof23pf/AEErP/v+v+NNOu6QnLapZD63C/40BdGjRWZ/wkGjAZ/tewx/18L/AI01vEugr97WdOH1uk/xoC6NWg1jHxb4cQZbXtLH1u4/8aY3jPwun3vEWkj/ALfY/wDGgLo3K858XHd8XPA8fol2f0X/AArpG8d+E1/5mPSvwu0/xrzzxF4x8O3PxZ8LXkes2j2dpbz+bMsoKqW6An8KRMmj2UUVy/8Awsbwd/0Men/9/hSj4ieDyOPEenf9/wAUyro6eiuWPxI8HD/mY9P/AO/tMPxM8GDr4jsP+/lAXR1lFcgfif4KUZPiOy/Bif6U0/FTwP8A9DFaf+Pf4UBdHY0Vxh+LHgYcf8JFa/k3+FMHxc8CH/mYYOP9h/8ACgLo7b60Vw//AAt7wGP+Zih/79Sf/E0f8Lf8B/8AQxQ/9+pP/iaAujuMiiuGHxh8BkZ/4SCIfWGX/wCJpF+MPgMk/wDFQRD/ALYyf/E0Bcb8Y3K/C/V8dwg/8eFdfpXGj2QHTyI+n0FeP/FH4k+Ftc8EXWm6Xqq3VzMy4VI3HAPOcgV1dl8XfA8Wn26vrkassSgr5MmRx9KCb6noVFcEfjL4EA/5DYP/AGxf/Cm/8Ln8Cb8f2z+Pkvj+VBV0d/RXn5+NHgUDjWM/SB/8KQfGrwKTj+1nH1gf/CgLo9Borz7/AIXV4FP/ADFz/wB+W/wpW+NHgUDI1gn2ED/4UBc9BpK88/4XZ4Fz/wAhST/vy1P/AOF0eBduf7YP08lv8KAuegUVwI+MvgQjP9tj6eS/+FM/4XT4Gzj+1mPv5D/4UBc9BqjrL+Xol++cbbeQ/wDjprjH+NPgdf8AmKO30gb/AArO1n4x+DbrQNRgt76VppbaSNF8huSVIFAXRq/Bnj4T6L/23/8AR8ld7Xifw6+KPhTw/wCAtL0vUL6SK6gRxIoiJxmRj1H1rqv+F1eCP+glL/34agSeh6FRXnf/AAu3wN/0Epf+/DUh+N3gb/oJS/8AfhqCj0XtRXnX/C7vA2f+QnL/AN+GoHxu8DE4/tKX/vw1AHogpa88/wCF1+Bhx/aj/hA/+FP/AOFz+Bsf8hZv+/D/AOFArnfnPbFFefj40+CD/wAxOT/wHb/Cj/hc/gfdxqj/APfhv8KAuj0ClFefH4z+CFOP7Tlyf+ndv8KUfGfwQempyf8AgO3+FAXR35rgfhQ/m6Rr83/PTXrx/wA2FI3xn8D7sDVWb6QP/hR8IZVufCV3eIpVLnU7iYZ64Ld6XUV9T0DAoooplHm2hn/i+HiH/rwhr0jFeb6G5Hxw8Qoe9hDXpIpIiGwUUUUywooooAMUUUUAHWijFFABQKKKACk6UtIaAPNtLwPjxrOeM6ZER7816VXm1iMfHrU8NkHSos8dOTXpI5pExCiiimUGPeiiloATHuaMUUUAGKMUtJQAYo7UtJQA3JrxL4Na1oll4Nu7TVdV0+1Lag8nk3VykZZfLjAOGIOMg/lXt+K4e4+E3gee5llfQkV5GLkR3EqKCTnhVcAD2AAFengcRhoUKtDEc1pcrvFJ7X7tdyJJ3TRxVn4j0i2+LWuXf9qWP2KSxj8qX7QnlM46gNnBNUPHGs6TfeFNWFtqlpLPIIsRJcoxfEqHgA5PAz+FTWvw+8OT/FrUdE/s/Omw2McyQ+fJ8rE8nduz+tdxD8HvBIXMmiEn/r6m/wDi66MNUyuhWhWTqPlae0ejv/MRabTWhueC0P8Awg3h88g/2bb/APota6EdKZBBFbQRwQRJFDEoSOONQqooGAABwAB2qWvIqz56kprq2zVKyEopaKzGJijFFBoACAeophiRuqKfqKfS0AQfZrc9YIz/AMBFRtYWjnLWsDE+sYq1RQKyKTaPpj/e060b/egX/Cm/2HpH/QLsv/Adf8Kv0UBY8r8H6Npx+JvjW1k061aKOSEohhUquUB4GOOtegf8I1oWSf7G07J7/ZU/wri/B24fFrxxn+9B/wCi1r0igmKVjIPhXw8xy2haYT6m0j/wph8IeGj18PaSf+3KP/CtqigqyMI+C/CxHPhvSP8AwCj/AMKjPgTwkTk+GdI/8Ao/8K6GigLI54eBPCQ/5lnSP/AKP/Cmv4B8ISDnwzpI/wB20QfyFdHRQFkcs3w58Guct4a04fSAD+VNPwz8Fnr4csP+/ddXRQFkcgfhd4Ibr4csvyP+NRv8KPAzHJ8O2v4Mw/rXZ0UBZHF/8Kn8C/8AQu23/fT/AONUdS+E/geHS7uWLw/CrpC7KRLJwQD/ALVehVS1T/kEXuenkSfyNAmlY8k+GXw38J6/4A0zU9U0hLi7nEheQyuM4kIHAOOgrrv+FOeAj/zL8f8A3/l/+KqL4MA/8Kq0bPfzcf8Af1q7+gElY4N/gz4CbpoKL9J5f/iqgb4J+BW6aS4+k7/416HRQOyPO/8AhSPgb/oGy/8AgQ1J/wAKQ8D/APQOm/8AAhq9FooCyPOv+FI+Cu1ndD6XLU3/AIUj4MxgW94v0uTXo9LQLlR5v/wpHwf/AM87/wD8CjSH4I+D9uBHfD3F0a9IooDlR5s3wS8KEjbLqif7t2f8KX/hSvhzGBqOuD6Xv/1q9IooDlj2PN1+C+gx/d1XXwPa+x/SuO8X/DfTNN8W+FLGLUdWlW/umjkM11uZABnKnHBr3mvOfGo3/FDwHGennzt+IiNAnFDh8HtGAwNb8RD6agf8KguPgrod06vcaxr0zp9wy3u4r9MivS6KB8qPOh8H9NUYXxH4lX6agf8ACg/CGx7eJvEw/wC4gf8ACvRaKA5Uebj4RWytkeK/EwH/AF/mnN8JVA+Txh4nX0/09jivRqPpQHKjzofCy4UEL468Uj6X7/40f8Ktuu/jzxWf+4g/+Nei0UDsjzv/AIVddf8AQ9+K/wDwYP8A40f8KvvAcr478UD63zH+teiYFFAuVHnZ+GWoEf8AI++Jv/As/wCNH/CstSxx4+8S/wDgUf8AGvRKQnCk9celAcqPN7n4Z3620xbx54lKhDkPdEjp9a5b4a+BbrWPA9jfQ+LdesFl3f6PaXJSNeewzXsmsvs0S/fptt5D/wCOmuT+D8fl/C3RMfxRM3/j5oFyq5WHwz1FTkePfE343ZP9aYfhnrOcr8Q/EQ57zE/1r0aigfKjzZvhjrp6fEbxAOf+eh/+KpR8NfEAGP8AhY2v/n/9evSKWgOVHnI+G/iAf81F1z8h/jR/wrfxAf8AmomufkP8a9GooDlR5x/wrjxCDlfiLrgPuAR/Oj/hXXiPP/JRtbx/uj/Gqnxn8Wa34b03TotIjubYTTiR9QTaUBXkRdzkkBjnAIUj5gWAZr3xttNCjtreTQL3+12ijkubOeQRC33Lu2l8ElsFTjaOG52sCo9Wjk2Lr0oVKK5ue9kmr6dX2/q+6IcoJtM0T8PPEPG34i62Pqqn+tA+HniMf81F1r/v2v8AjWVq/wAeNFs7K0m03Tbm8muF8wxSypF5S7nXDFS5DZQHbj7rA57VjeI/izf3/wDwiWo+HYL1Ee5cXdku0+fKuwGAHBLfLJwduP3iEfMuF0pZBj5tKUOVO+r7pN+vQHOCOs/4V34j/wCij6x/36X/ABqC68Ea1Z+T9q+KOpwedKsMXmhF8yQ9EXLcscHAHNekQSNLBHI8Lws6hjFIQWQkfdO0kZHTgke5ryfU7ODxn8ef7L1GPfYaFYib7NIS8c7na2dvAXmVM9dwiAPBwOPB4WNec+d2jGLk7a7dvVtIqTS2MHR/ButXXxQ16zTxjqMdza20PmXqKPMkDdFPPQYrtf8AhXviX/oo2sf9+l/xryXTp9e8X3/jLxPputXOk3FrD9seGGVk8yIFiIy6Y+6qnGRyeuMk17x4I1m68VfD/TtRnkeC7uIGjkmj2lt6s0ZkAK7QSV3Y2kDOORXTjcqlhIc7mnZ8skr+62r28/VERakzEHw/8S85+Iur8+kKUz/hXniQHI+I2tf9+1/xrgvF2i+JfDOraNpEHxE1a91LVJ1ijiaeSJYlLBQ7kSswBY4Hy84bnjBj+ID+PE8falaaNdeJp7eGK3Km1Mu0gxKN+IwFG5lfoAMhvQ110shjVceSurSTd2mtml1t1f4EuaW6O6l8E61b3VvayfFDU47m43eRDJs3y7RltoLZOBycdKn/AOFeeJe/xG1n/v0v+Ncv4psLLxJ8JtO8UaRqdzqGr6KsZOoGPF0QpG9H2nKlCwfJ3EBc7juLn1vw/rEWv+H9P1aHYFu4FlKJIHCMR8ybh1KnKnpyDwK8/FYH2FJVE76uMtLWa/HVfqXGzdjiz8N/EWMf8LG1z8h/jR/wrnxJgD/hY2tf98D/ABr0eivOL5Uecf8ACuvEv/RR9a/79D/Gl/4V54m/6KPrP/fpf8a9FNGKA5Uec/8ACvPEuf8Ako+sf9+l/wAaUfDvxGP+ai61/wB+1/xr0WigOVHnX/CuNfb73xF1049MD+tcP478Eanp+reFIbjxfqt9Jd6msEcs7c25OPmXnrXvtebfEr954t8AQDvq/mf984NAnFIefhrrX8PxD8QAn1kz/WgfDjX8Y/4WLrv6f416NRigfKjzpfhvrgzn4h68c9eR/jTx8OtbCYPxB18nudwr0KigOVHAD4eaxjH/AAn2v/8AfQpn/CuNXOM+P/ER/wC2tehUUByo88Pw21U/8z/4j/7/AFKnw01HGH8e+JW+l0RXoWKKA5Innv8AwrG97+PPFH/gaab/AMKuu+3jvxSP+35v8a9EooDlR54Phhd4wfHfir/wYN/jS/8ACr7g9fHXiz/wYNXoVFA+VHjfjj4e/wBl+C9XvpPFfiO7EFuzeRc3zPG57AjuK0fD/wAMWfw/p7N4u8TRh4FcxQX7RoMjOAOwroPiqwj+GWu5Gc25H5muj0EY8Pab/wBesX/oIoJ5Vc5Jfhei9fGHi38NVYU0fCyDPPivxUf+4o1d/RQPkRwA+FGn458R+Jzj/qJt/hQPhPpuMHxB4mP/AHE2/wAK7+igORHn3/CotI/6DniT/wAGTf4UjfCHQ2H7zVNeb3bUW4r0KjFAcqPPf+FPaBnJ1HXSw6E6g2RTh8IdAzk3+uE476g1egUUByo8+/4U/wCHSuHu9ZcH+9ftSL8HfDG7cz6ozdyb5+a9BxS0Byo85f4KeCyGaW1u3Pq90xrFb4LeETKxFpdBSeP9IP8AhXrky7l21AluqsWI4AoDlR4V8M/hh4b8RWGsXeqWssvk6jJbQr5xUKigenfk16CPgt4EXn+xyfrcSf40nwijx4Xv5+P3+q3UnH+9j+legUCjqtTg/wDhTXgI/wDMBT/v/L/8VQPg34CXn/hH4z9Z5f8A4qu8ooKsjhR8HfAQ5/4R6I/WeX/4qpB8IfAf/Quwf9/ZP/iq7aigLI4ofCXwKhyPDlt+Luf61IPhT4GGf+Kbs+f97/GuxooCyOQT4XeCIxhfDdif95Sf5mpP+FZ+Cv8AoWdO/wC/Irq6KAsjlB8NPBQGP+EZ07/vyKUfDbwWOnhnTfxgFdVRQFkcwPh34NH/ADLGlfjar/hXB6r4S8On4z6Jp0eh6elm2my</t>
+  </si>
+  <si>
+    <t>/9j/4AAQSkZJRgABAQAAAQABAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCARDBdwDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD3KGaMW0ciRSKGUbVKHdjtkdvxrnrLx1a3uGj0bXlgaPzIpzpsnlyjGQFwCfzAra0+SY2wilbdJDmORliaNMj03cnqOckHBrnfhg9zN8PtJkuZ3nmIlEkkj+YxYSsPvZ5Axj8BQDLOp+OtM0eKwlv7a/gN67hEkgw42AE5BPuMAZJJwBmqU/xItEKNZ+HvE2owugkW4tNJk2HOeAWxz+nNdXeypbRvOzoD0HmzlF/rz+FVo7uO4giSG+/eyLxIgzkc9M8Z470BZnEH4iiaa3EngTxdAIGymNJB2jGM89Pwq4/xEa4diPCHjMCMEhRphXzOPXP+FdgbopNsQu5IByVwOQccn1I7Cp4w20NIR5vDMqucE4x+VAWZxFr8SLdYwX8I+L7ePjMsulMc8YGSCSe3NIPizZssuzwr4tcRZ80rpf8Aq/r83H/1q7su5fPCqh+Y/hTROWwyAMDgj5ucH2/z0oFZnERfFKxkuBEPDfisxgbzN/ZZK7cZycHOOfSi4+K2gg8Wuu/K21wumv8AJ9cj6V3vz8EYx3GKYAQo+due5AzQGpwo+KvhZkjG7VyHfC/6BPkt6ZA5+lK3xj8GxkLJeXqE9A1hMD/6DXdbwvDuoP0xinkkEZxigNTgG+NHgfZk6jdAHv8AYpv/AImkHxr8CZx/aswOf+fKb/4mvQAeM9R60EknAH40Bqefj41+ANuTrbgjsbOfP/oFP/4XV8Psc+IP/JKf/wCN13xJHp1rzT43yxx+AoVkgjkMmoQKnmAHack5H4Aj6E0BsXf+F0/D3P8AyMH/AJJXH/xFB+NXw8P/ADMH/klcf/G67iS1tpCplt4mx0LKDg0hsrVnLNbQlmOSSgyaA1OJHxo+HzDP/CQDj1s5/wD4ipT8XvAAZQfEEOTwP3EvH/jvFdZLpenzoFmsLaRR0DQggfpVY+GtBLhjommlvX7Kmf5UBqZFr8TvBN4haLxLp6gf89pfKP5NirX/AAsDwb/0NOj/APgbH/jVtvCnhx/vaDpZ+tnH/hUB8FeFWOT4Z0Y55/48Yv8ACgNSP/hP/Bx5/wCEo0f/AMDo/wDGnf8ACeeD/wDoaNF/8Dov8aX/AIQnwn/0K+i/+AEP+FH/AAhHhIn/AJFbRP8AwAh/wpBqH/CdeETz/wAJTon/AIMIf/iqX/hOvCJ/5mnRP/BhD/8AFUxvAng912t4X0YZ9LGIH+VRv4A8Hyo6t4X0cBuDtsowfzA4/CmGpYHjfwocAeJ9FJ9r+L/GrA8UaAz7F1zTS/XAukzj86xZvhd4JniEbeGrEADHyKVP5gg1Wf4P+ApHLt4eiyf7s0oH5BqQanbCaJhlXU/Q07zE/vD864I/BT4enk+H/wDycn/+Lpv/AApT4e9tA/8AJ2f/AOOUwO+3p/eH50BlPGR7c14N4D+G3hLWdd8YWt/pbTw6bqTW9sPtEi7EBbjhhnp1Nd1/wpP4ff8AQBb/AMDJ/wD4ugNT0AAE54/Clx7V5rcfAvwNKx8qyurfI/5ZXTnH/fRNVm+AXhItlLrV4h3VbkYP5rQB6nz2oxXlSfATw5GpVNa8RIhOSFuowP8A0XVyL4O2cUPlReMPF0ak52pqIAz642UBqek4pa86/wCFUnjHjvxkP+4p/wDY0f8ACqWB/wCR88Zf+DT/AOtQB6LiivOm+Fc+Pk8feMR9dSJ/pVE/CvxBg4+JfiMHnGZW49P+Wn+fagLnqeKK8p/4Vb4uRcR/FLWQe2+Jm/8AatTJ8O/G8Spt+KN8dhyN9gG/PMnP40Bc9Qo59K82Hgbx6rAj4nTfL0zpUZ/9mqT/AIRT4kDhfiTGfrokFAXPRRQTXiiSfEl/iHL4S/4TmLdHY/bftP8AZcOCNwGNuOvPrXQTeGPikBmHx/ZsfR9LiUfyNAXPS+1GOMV5dJoHxeTiHxnpMvvLZKv8ozSrpfxmQ/8AIweG5R/tRMP5RUBc9QxRj8K81jtPjHF97UfCUv8AvLMP5KKlH/C31H3vBr/+BFAXPRaO/SvPTL8XVH+p8Gt9Dc0w3HxeHS08IH6NP/jQFz0WjFebm9+L6/8AML8LN/uyzf1NV21n4xIT/wAUxoMg/wBm4I/nJQFz1GkrzCHxF8WlGZ/AumyH/pnfxpj85DU//CVfE4dfh1Bn/sLQ/wCNAXPSKTFedf8ACYfEVThvhrn0xrEP+FB8a+PgcH4Yy/hq8R/9loC56NniivJ9L+KviTWLu/tLDwBPNcafJ5Vyi6kn7p8kYOUHoelaL+PfGcQ3P8M77/gN+jfyWgLo9H6Vk+J7OfUfCes2VrH5lxcWM8USZA3OyEAZPA5I61w5+JPixT83wy1fn0nz/wCyVw/xE+JHii6h06E6ZrPhaMO7u28q0+AuNrAKTtBORnB3DPQV25dQlXxMIRaT3u9tFfp6EylZFG68MeJNV+HmgxS+GNTWPQrmeOeHaUnuY5nV90aFSwxypO0gZBG7DBatt4F1BtD1a/PgfVmh8+3jt0muWW7hUHMpVBGBIGGF3FPl3AgNtYjl08da/K0ix+KNfJHK5unwenX95x39ew78e06f8W9YGk2O/wAD+Ib+X7NEZbpLYqkzbRl1AUjaTyMdjX1WIzmdDDqrQcZRcntzqzupNa23b37O22hgoJuzOI8O+BvEOo2fii0stAvNPt7ixjEK6moEjSLNG4QSFEJyEk6ALnbu6A17H8NdS1K98J21pqWg3ulSadFFaKbkY88JGo3gEBh09McjBPOMSH4uSHIuPAviuM4HCWG7nv1Iqb/hb9qP+ZN8Y/8AgrH/AMXXg4/OJY2DhOCWqa3utEn11ul1NYQ5Xoyj8ZP+Jdf+D/Ec3zWem6mPOROZGyUf5QeDxC3Ujkj8Kmux694Z+JUvjfQtHfxBpeq2ccTC1+YjKrjaU3HH7pG37duGx1wau6n8T9G1fTZ9O1HwN4tntJ12SRPpgwR/384IOCCOQQCOar6F8RtE8N6Ha6PYeD/GQtrZSq+Zp4ZmJJJYnf1JJPGBzwAOKdDNIUsPGm43aUotPZxk77p3TTBxu7mLoTeNvDHh/WPFVtoLy6vrmqqX097KVjHGBKzSbFbeoLtgbugAPO4Gp/E+mappPxKu/Etx4HfxDYanZoI7UxiU27hYwd4VXAYbCOMghuGOCK6T/hcmmg7f+EX8VZxnH9nD/wCLqKX426FA5SXQ/ESMCAQ1kARnp1bvVf22/auq6a95NPVq60srp6WstRcita55tY+AvEXh2z0LWtS8PXOt2hnklfRU3ExEouxnUAkFioJG0jEaq3J2jsfBjXuja54m8bajob+G9AFmE/s0/ut0ihMbEIQEnDAEgZaXAzlsabfHvwqmd9hra465tV4/8frD8S/Fj4d+K9OhsNYsdaa3WdJ12xBDuXtkP0ILKfZjjBwRvUz54q8MRGylo2r/AA3vZRva/nuJU+XY6L4LaZP/AGBqHia9uPOvNduWmcjAGEZxkgAYYuZDxxjbjHNem968Gn+PdjaeKNNt9NsfL8MxwiGdGg8uSPkgFApICqoXA78+2Ovg+OfgSWMs9/cwnsslq5J/IGvGxuJeKxE6zVrvRdlsl8loaRXKrHpQo6V5yPjf4DMpjOrTAD/lobSXB/8AHc/pTh8bPABcqdacADO42k2D7fcrlKueiGjtXn4+Nfw/Iy2vFcjobOf/AOIpf+F1/D3/AKGH/wAk5/8A4igLnfk4orgf+F0/D4/8zAP/AAEn/wDiKX/hc/gD/oYU/wDAab/4igLne4pK4UfGPwCf+Zij/wC/E3/xNOHxh8BE/wDIxQ/9+Zf/AImgLncjmj6Vw3/C4PAWAf8AhIoeeP8AUy//ABNOHxc8BscDxHb/AIxyD/2WgLnbUuK40fFfwK3TxJafjuH9KX/hangb/oZbL8z/AIUDOx70Vxw+Kfgc9PEtl+JP+FSD4neCSM/8JLp//f2gVzraO9covxK8Ft08T6b+MwFOX4jeDGOF8UaX+NyooC51GOODSKCFAJyfWud/4WB4O/6GjSP/AAMj/wAaUePvCBwR4p0b8b6If1oC6OjqreW63MBVoY5SpDqr9Nw5B/A1kf8ACeeEf+hp0X/wPi/xoPjvwiOD4p0Qf9v8X+NAXHeH/DWn6BLey2dlFby3MimRo1xvAUAf/X98mt/Fc9/wnnhA8f8ACU6L/wCB8X+NH/Cc+ER/zNWif+DGH/4qgZ0Bo71g/wDCd+Ef+hp0T/wYw/8AxVNHjrwhj/katD/8GEP/AMVQB0FH4VgDx14RH/M1aJ/4MIf/AIqg+OPCI4PirRB/3EIv/iqAN+jGawP+E68I/wDQ1aJ/4MYf/iqP+E78If8AQ1aH/wCDGH/4qgDfAwaK5/8A4Tnwh/0NWh/+DCH/AOKo/wCE68If9DVof/gwh/8AiqAOh6jFJjFc/wD8J34P/wChr0T/AMGEX/xVL/wnXhH/AKGrRP8AwYw//FUAb+KOprnf+E98Hscf8JTov430WP50h8e+EFJH/CU6NxzxfRH+tArl7xNq39heGNU1QPCr2ttJJH55wjSBTsU8jOWwMA5OcCvDPDvjPx54is7u4Txxo9gLXBlS/jijbaSAGH7kgjJA65BxnGRn0vxN458Kaj4W1iwtfEelyXVzYzxRJ9rQBmZCANxIA5Pc18wfasWf2fzHCNIH2hwFY4IBIx8xGeDnjLY+8a+t4ew9Gth6l4xcuZatRdl6P+mzCrKzR9B/Cz4iXWrQ63H4n1qwdbJo3iuZNkG5GJVj0UbQdmCQDl8HqAOoHxO8L3Wj6tf6ZqcN0+nWzXDQSboC/ZQC6jOW2rkA4LL6jPzFpM2nxR6kmoz3say2brCtrIi+ZLuUosgY/NHuAJAyeAR0rS0e60bTNZuPJunmt59Nu4FnvoRbmOV4JFXaFkYckhcscfOeBgGvSxuQ4J1KtVtrls7KyirJXv2v8t9LkRqyskfSfgDxpb+NfDkd7mGPUIvkvLaNj+7fnBwedrAZHXuMkqaj+JXiiXwl4Kur+0lSO+kZYLUvGXG9jycdMhA7DPGVGc9DwPwq+IvhHRfCEGk390unXcJeWWWSMBLgs7EEMuckLsB3YPAxkDiD4xeM/DfiPwja2ej6xbXdyl8kzRxsc7Ajgnnrywr5/wCp0Y5yqEo2hz6J9unyfTy03NuZ+zv1KFnZav8AC7VtJ0/Qd+o+JNZs0N1p0wJhhO4nOFIDEYIDbsKEkJ4cbfQ/AHjrVde1nVdA8SafDYazY4kEUKsA0fAPUsOCVIO7DBwQMDJ4DxX4/wBBi+Kvh/xXpt7HqVpb2pgmhh3JKn+sBOGA7S5AzyVIO3rVHTfiTYW3j/xL40EKDzrZLe106WYrLP8ANEu7IUgYWIsfTIAz1r1a1CWPw3tZwTlKPxbP2nPZQ7LTTVfPqZqXK7J/8MexeP8AxnB4K8OSXuYZNQl+SztpGP7x+MnA52qDk9OwyCwrmNU+KOoWfwm0vxVDp9t9uvp/s5jdmMSMDIGbAwSD5ZwM8bhycc+a+O/ENp4uvo9ai8VaasaWPy6VdRyFraRo8SRp+6KMxPSQ7TnHTaprCh8Q3DeFtM0W+8Ro+hi6Hn6VZrtuUTezMSSgVu5ALkZK8ccRgsrwToU+dxc+dcybd9n7iXfT5u+trDlUld9j1nw/468R+LdSu/CmoC2srm8s2e31LQ5UnFrjOTIRI4APAyCrAkYwWDCT4I2cEP8AwkRv493iWC+aG9lkJeQIe2/kHMiyE4PJAJz8tcZ4f8b+FdA+I9pdaEbrRfDc1qY7+G6JfzJAJCrY3OepjAI5HPYnOh4S8f8Ah3T/AIkeKdd1DV47Cxu22W9vDbSbLkbuJioBw2FycjJMrHjkUY+EKVGvThHkjywduvNe1mtbXWtrtaJ9xRbbTep790oz7VwH/C6/h6P+Zg/8k5//AIij/hdXw+/6GD/ySuP/AI3Xxx0nf9Bmlrzx/jX4AC5XXWY+gs5/6pUEfxx8CtGSdSuVIz8rWkmf0GKBXPSKWvLz8evBQTdv1E+gFt1/WmSfH7wcrBY4tUmJ/uWw/qwoC56maK8uX48+FnbbHp+uOf8AZtAf/ZqnT41aE7bE0TxGz/3RYZP/AKFQFz0rFHtXnLfGDTx08LeLG+mm/wD2VM/4XFY/9Cn4t/8ABaP/AIqgLnpVJ3rzkfF60JAXwf4vJPTGmD/4unD4tW7Z2+DPGRxxxpY/+LoC56JRXnb/ABUmwPK8A+Mm9c6Zj+pqA/FXUyfl+HXir23WZH9KAuj0uivM4/ib4gmB8v4b+IBgfxrt5/FaUfEbxY33fhnq/wDwK4A/9loC6PS8ijFeWaj8UPE2lafNf3/w6vbe0gGZZXvlwozj+771NZfETxhqNnDd2fw3uZbeZBJFIdSRdykZB5WgLnpuRQefavOh418eN0+GU346xD/8TR/wmfxAJ4+GMn/g6h/+JoC56LRXncniz4imMmL4bBW7FtbhOPwwKZP4n+JzgfZvh5bRHv52rwvn8iKAuej0ZFeXS6/8X3IMPg7R4hjkS3YfP5SClj1f4xPnPhzw9Hg/xzn+klAXPUKK8yTUPjC3XRfDSfNj5pn6evDdP1qwLj4vMP8Ajy8Irzj5nn/oaAuei0V5153xgzxbeDh9Tcf404SfF8nHleCx/wCBP+NAHoeRRXnUifF+UAibwZFg/wAIuefzBrmvFF98XPCugXeuX+taA1rbbd0dvES3zMFGN0Y7sO9AXPas8Zoz7V5Na6X8Y7q2jn/4SjQkWVQ6j7PkgHn/AJ5Vag8PfFl3X7R430yNcc+VYI/80FAXPT8ijFedHwv8S2OR8RIF9ho8NJ/wivxK6n4jw/8AgmhoC5397eW+nWNxe3Unl21vE0sr4J2ooJJwOTwD0rwTUPG/w21Lxivia407xEbsrtlhUReTN8hT5135IK4BUEKQMEEE56nxN4b8fW3hXVprvx8t1apZzNPbjSYU8xNhyu7ORkZGRyM14nF4w8T2eipotpq7rpJgeN7YRx4Cuzb1yRuOck56jPbivocnhGFGVblk25KHuu2jTb6PsZVG27HtvhX4XeBNYSx8T6f/AGhPZTMZo7K6dTEpBI2Mu3cQrAjBYg7eSwPNo/Anwj9v+0ebqflebv8As3nr5e3Odmdu7b2+9nHfPNYXw78L+LdS8C6ddad45l0yyfzfLtE06OXy8SuD8xOTkgn8a6geCvHORu+JlyfppUI/rWONzPHUMVUpwrStFuO/RN2+fmEYRcU7GrJ8ONAbxrF4qiFzbXyN5jR28vlxSPggswAzk55AIDdwctnqp4IrmCSCeJJYZVKSRyKGV1IwQQeCCO1eat8NfFBkmc/EzWczAhtsWAMnPA34X8MVCPhP4g3Av8TfEhHcLNIM/wDkSvKq4irV5faSb5VZeSNEkth/gfwpq+lJrXgfxDp6aj4cK+db3rMQrBz9wLnKnILYGCjAnJ3K1anhj4S+HvCuuRavZy6hPcxKyx/aZVKoWGC2FVcnBI5yOemcEUB8KdSzz8RvFmPa+b/GrP8Awqqbv4/8Zn/uKH/CuytmuJqObUuVT+JLZu1m7efWwlCKOg8H+CtN8E2FxaabPeSpPL5rG5l3YOAOAAFHTrjJ4yTgYtaN4X0vQdS1a/sInSfVZxPclpCwLc8AHoMszfVj2AA8q8f+EL3wp4ZGo2PjbxXLObmKELPqTFfnbB6AV1Q+FBxz488Z/wDg0/8Asa5KmKrVJSlOTblv527jUUjqrjwtpd34qs/EksT/ANpWcDQROshC7WzyV6EgM4H++c5wMcf4M0DX9T8c6l408TWiWUm1rOxsXPmNAoIBZWJwowGGR9/e7AAEbpx8KR38deND/wBxX/7Gg/CmMgg+OPGpB6/8TXr/AOOVrTx1WFOUN7rlu91G92l6/wDDA4pu56EOfajB9eK8qk+Anh2Zi0mu+I3Y9S13Gf8A2nUZ/Z98LEjfquvN9bmL/wCN1xjPWsd6PevN/wDhSPgkbsWd5zgf8fb8Y64579/rxip/+FLeAhx/Y0v/AIGz/wDxVAHf7h6ijev94V5//wAKS+H566GxP/X5P/8AF0f8KS+H4/5gLH/t8n/+LoDU9A3r6j86TzUHVl/OuA/4Un8Puf8AiQn6fbZ//jlKPgp8Psf8gE/+Bs//AMcpBqd2biL/AJ6oOP71N+1264DXMWT/ALQFcMPgr8Pj/wAy+R/2+z//AByuK8efDXwjouo+FINP0jyV1DWIre4X7TM3mRHqOWOPqOaA1Pbje2wPNzCPq4qGXVtPgjMs19axxjq7zKAPxzXHD4MfD5CSPD4P/b3Of/Z6l/4VD4A6f8I9Dz/03l/+KoDU6P8A4STQzaLdrrOnG3ZiizfaU2kjqAc4zwarv428KRHa/ibRVPob+If1rET4QeAYxtXw7CeO80pP6tTh8I/AXbw5B+Msn/xVMNTXPjnwiD/yNWiD/uIQ/wDxVA8d+Ee/ivQ//BhD/wDFVl/8Kq8CtGU/4Ry0xnr82ePfNXE+Hng1JI3XwvpJKR7Bm1Ugj3BGCfc80DJ/+E78IHj/AISnRP8AwPi/xpT468I4/wCRq0P/AMGEP/xVH/CC+EP+hV0P/wAF8P8A8TQPAvhH/oVdD/8ABfD/APE0CGf8J74PH/M0aN/4HRf40f8ACwPB3QeKdH/8DY/8ak/4Qjwp0HhfRAP+vCL/AOJpf+EJ8Jgf8ivov/gBF/8AE0BqRf8ACwfBv/Q06P8A+Bsf+NH/AAsDwd/0NOj/APgan+NS/wDCF+E8Z/4RfRT/ANuEP+FKPBXhTH/Ir6L/AOAEX/xNAxLu1vJvDN+q+VLqEltLGjhOGJBwOp4yfX8qy/DVinhnwPpmkC6sZp4B5TEP+73GQmTA6nBz+XarfiVCvgLXIorVnf8As64CwheWPlnAGOv4VQ+HkemW/wAPtAOniMQPbhz5shypYkyAZHOGLCjqHU2ZrOztbgX8geWbcZVVcsxOMcc9OfpUhe4W5Mgsl8122BjLwqjkEg9u3Hcj6ifM7XZC2iBY8qkrsMgYB4Azxnjt92n7ZxBJ9oaB+MBiOOvp+XfrQUQQzrGHldgTtGWkbk/h/nrUxREjUAy4c5KjOc5B69qZLJCjyM95Fg8gO44GBkfT6561aCrGRyd7cDIOM0xCMXwwQjO8Ahhng49/enBiFK8EkYAHH/16ajHeQytlBkHsRz39fWnEsAPkAX1zmgQBmWUrs2qehAzk4708kj5Qucdyaqw3kVxqFzaBG8+12lgRgEMDhh6jgj6g1aUBUBVeF7Y5/WkAql+QwU+hHej+LAznqfSgkjnkflS8kkFTx0JPBoAO/wBP1p/4/jUfVcvgcc4bpSqVKAqcrjqO9AAWwRnuccV5v8arb7b4S0qDesXmaxbr5jc7M7hn9a9I4w3HGfTrXmvxqAk8O6BG7mNH163VmHYYk5oE9j0w43e4FHTjH/1qacAgnqadk56UDA/hTehA5P8ASndceuKCMnk/hQAEjufalz7UlGfcZ9KAF4NGQD1o70A0AJz6flRx6Ue9L6AUABzRSYPP+NL+HFAB1oxigdKOvPNAHmHwrx/wlPxCxx/xPJP/AEJ69P4rzH4VZbxJ4/Y4512UfkzV6dgnqaBITP0pfekIGMjFAPH+FAyMTRPcPAkqGZFV2jDDcqsSASOoBKtg+x9KlrwG1n8SaN8ZvE+ozXlncXGn2Mt3ehYiqXFsqIyxoOSjY8oZycYJJfBDUdI+NfiubxPbtcxw3NncSxxNYW1rkgEqD5XO4ucHAZiMt06Y+i/1crzXNQkpLlUu26vZfptoY+2S3PozNMjmileVI5Udom2SKrAlGwGwfQ4ZTj0IPevnKD4x+NI/Fcf2v7MkSziKbTJI1gjB+6yl3+ZDnJyzYB68DFdV8LYdX/4WZ4zf7ZbfZI7yRb1BCQZpDJJsZBklACH6s3Bxgn5ljEcP1sNRnVrTStFNW1vqlb8fRvruNVVJ2R7MDXMaP4+0DXdS1a0sbh2i0tQ894yYtivOSJOmBg8nGcErkAmtLxNd3GneE9ZvbVxHPb2M80T7QdrrGxBweDyB1rwi/wD+JZ+zlpn2P93/AGpqbfbO/m4aTHXp/qY+mPu+5zjluXQxVNub1lKMV5Xu2330Wnmxznys970/xBourztBp2r6feTKu8x29ykjBcgZwpJxkjn3qbUNU0/SIFn1C9trOFm2CS5mWNS2CcZYjnAPHtXjWveFNN8AfEHwJN4f86GS6uRbTmR/M8wbkRm5HDMsrA4wOmAK9U8T+HPD3iGwU+IrSGW3tN0wlkkMflDHzHeCCFwMnnHAJ6Cs8Rg8NSlSnGUnTmn0XNo2tr23XcFJu66otaf4g0XVp2g03V9PvJlXeY7a5SRguQM4Uk4yRz71civbWe8uLWG5hkuLfb58KSAvFuGV3AcjI5GeteOfBvRNN1DxHrniiz077NYRS/ZdNjZt2wHlidxZg+3Zk5x+8cDjgHw/0YeHfjl4i003k135diz+fOcyPveF/mPdvmwT3POBnFdOIyqhCpWhCbvTipWa66XWjtpdL19BKbsnbcs+E9ag1/8AaA1u9tUuFhj0l7bE8RjYMksan5TyOR0IB55Ar2AD3rxG/wBaXQv2k1ZPMEV8sNpcBFDbzIiqvXoA6xk45wO+cH26uHH4aFL2dSlflnFNX6PZr719xUHe6YYpaTvS155YlFHel6UAHWkpe9J1oAWjtQKKACiikzn1pAFFLSEdKYHl/wAJ7YjxD4/v+qT69LEP+Asx/wDagr1DvXmfwpgkGr+PLreTHJ4gnRVPQEMST/48Pyr0ygSA15j8W/CeteJG0K60exgvzYSyNNbTSBQ4bYRnJAK/Jg8g8jHcj07mkHXNdOExU8LWVaCTavvtqrP8GKUeZWPmu6+HvjNlulg8E6fZG8hWBzbXC9A6uMAzEA5Qduma+gfDunT6P4c0vTp5FkltbSKByhJXcqBTjIBxkelamMnJHSjHetsVmEq9JUVCMIp391Pd6dW+wows73FooozXAWGaKMUlABnrRR26UtADea82+M4LaBoCgAhtetQQe/EnFelV5z8YQW0zwuo6t4jtB+klAmejc9hTSoJyVH1Ip3OenFHagZA8NukZZoI8AZ+6Kb9gtGwTa27HsfKFWSMgijGOgoArNp1kxJaytyTySYxz+lN/svTj/wAuNr/35X/CreM0ooApnStOz/x4Wv8A35X/AApDpWmj/mH2n/flf8Ku0c0AUP7I0xs/8S60/wC/C/4U1NC0iMkx6VZAnri3UZ/StDBpaBWMpfD2ix7ymj6epk+/i1QbvrxzTZvDOgzx7J9E06Rf7rWqEfyrW5paAscT4t8KeGrXwdrVzH4e0pGgsJ5VZLKIFSIycg44PFZHw98M+Gpfhlo9/e6Bp9zJ9lMksjWCyyPgsf7pZj7AEmus8dA/8K98S/8AYKuv/RTVW+G8H2X4beHYz3sIpP8Avobv6015hbU8v8HeLPBmq6zrq614b0a206PNzZS/2TH+6hX5SshUH5j8mOuWYqDyi1v6V4n+E2rXl3aR+H9Nh8hZJFebSE2zIis7uu1ScBUJwwU8jAzxXPzeGfE1xqnxC0KLQbnGsT/are8chYcRzmVV3n5SXV8DByGwCANxXm/DngXUL3WLMP4H1aSKCCSS8i1G5a3iuGCYUI/lqUO7ouWzkZIAZq+1nlmV1lOo3y6KyUo/yp31tu7rXqr6Xuc/NNWR32l+JvhLq+svpsXhmxjb5vKml0mLZOR0VAoLFm/hBUE9MbiAYPhTL4b8Z2t/b6n4T0X7fbSmTfDpKLF5TH5V3YIDA7gAcEqAfmIY1xnhHwrrMPjLw5LbeFdZtGhuY2vJr+INEVBBZlDRKEwA5GSxztwdwGfQ/hPa694Tvr7wlqfh+5EInkuf7UjOYD8qKACQAQQM8Etk4KjDEYZhl2BoUKsaGsrRavJXVm02vXTTqEJSbVzW8ceHfCPhzwVq2qx+F9JWaGArCyafCxWRyEQ4IwQGZSfYHg9K8vufD1p4c8B+HIrXSrO+8S+JJUeKe5gjmSKP5SqJ5g2qT5kYOQRy/PC49k+KGny6l8NdcghZFdIBOS5IG2JlkYcDrhDj3x0rzy+tb/xP8PvBPiLwxD9tvPDu1JbMhS26NUySA2TzCuFHzMJARiufKFSWHjz2s5tSvtpG8E/Jy+RVRO+nYq+F9ATSfiMvhPxhoWhXxvbbzbSa3sIQoIDNnKqp2kK4OVzlRjg5PT+MfhZLez2h8J2HhqwhVWE6XGnoWZsjB3GNxjHbAx6nI24tpJ4s8SeO7rxnN4budLOjaVKLO2ngdjcSeXIEj52sxLOx+UdAF6kE9Bq2qeM/EPwkbb4fmh1u/lNnPCEEWyJnKlwjknaVwp3YI3F+FANPE4e2JpVIqmnaKkvd5VJ36baKz06gno1qeT2UqWng3XNYvdL0S+jNymnafcLpcIXziGZnHCEKIxkBkOSycDDA7Fn4YufDfi3QtO8Z6JpF1Ya2vkBbe1iV4pGwuNyBCGVmTJBIwx2kkcdt4i+GF0PhFZeHtJRJdStJ47uVUKj7TMQVf5ztGAHOCedqKKyYpPFnxD8c+F5tU8N3OjW2jt9pmnkgdVdwVZsb9vDFEUKMkZJJYDjtU8FWjOpThBQvPm0Skkorkceur10W5NpLRkXgXwboFp8QPE3hLWNLttSa2C3NnLNErlYuOGbAO4rJFxjGQ2Md/Qb34deDI9PuJF8NaaCsTEHyBkcVyvhl08a/GrVvEUV15lhocQtbTaV+YsGTIKghkJ85gc5+ZO3A9K16b7N4e1OfP+rtZX/JSa8DOV/tClL43GLl/ia1+/RvzZrT2PMvhR4G8Mat8NdJv9S0Kyububzi8sseWbEzgfoBXZn4a+CQP+RY03/vyKofB1cfCfQsf3Jf/Rr13VeSWcoPhr4LU5HhjTfxgBpx+Gngon/kWNN/78Cup6jmjtQOxyw+G/gvkjwzpnP/AE7ilb4c+DGOW8MaX+FsorqKUUCscqnw38GIwYeGdMyDnm3BH61MPh94OHA8L6Rj/rzT/CukowKAscyPh/4PDZHhfSPxsoyP5U5PAPg9OR4W0c/WyjP8xXSUlAWPIvizpmieFfCEV5o/hvQobme8jg81tMhcopVmOAVIz8gHIPBPfBHC/Di7k1bxxpmma34e0aW0vo5CEn0W2jO1VYh1KoD1jI5yMZ46Ee9eK/Cmm+MdH/szUzMIhKsySQPtdHGRkZBHQsOQevrgjA8MfCXw94T1yLWLOa/nuoVZYxcSqVQsMEgKq5OCRzkc9M4I97C4rAwwMqdSK57S+ym7te61Lpb+vPOUZc11sTeJfB3hW08Kaxcx+G9GieGymkWRbCIFCIyQc44xWD8KPCHh+9+Gej3WpaBpl1dSiVnmntI5HYea+MkjPTFdn47bZ8PvEh7/ANl3P/opqZ8P4kg+HfhtIxgHTYGP1MYJ/U14Jp1JP+EF8I9f+EW0P/wXw/8AxNJN4D8JTQywt4Z0lVkUqTHZojAEY4ZQCD7ggiuh6dqWnGTi1KLs0OxxXhn4ZeHfDumS2ctnb6mZJ3l869t43cKeFQHHQAD6nceM4G8vhjw+n3dD00duLRP8K1qWrq1Z1pupUd29WSo20Rljw5og6aNp4B/6dk/wo/4R3RR00fT/APwGT/CtMEEnjpS96zHY5zxB4N0vXtAvNMiiisXuI9i3NvCoaM5B9BkHGCMjIJGRnNT6F4R0Tw9pMOnWNjD5UY5eVFaSRu7M2OSfy7DAAFblLWvt6nsvY39297eYWV7lT7BZ9PsVv/36H+FOWytVPy20A+kYqweKKyGRLbwKciCMH2UVgeOhHH8PvEhAC/8AErueg/6ZMBXSVxXxauWtPhbr8qnloBF+DuqH+dAi/wDD5fL+HfhsY66bAfzjBrpqwvBkRg8DeH4W6x6bbKfqIlrd70Ag70Ue9JxQMWigACigDyvWvis+mfFa10FYZjpcf+jXS/ZGMrzP91kH3mUfJjA+YMxAbKGtW6+M3gy01kaeb2aWMZD3kMJeBGGeMj5m6cFVIO4c9cZXjK01mx+MnhvxDZaHe6lZx232ZzbAHaxMitk9FwJQcttB55GCR5PcfDvX7Ke40iTwzq1zqQnEcN7bPm0Kkrg8x4IIz8xdcZ5A2kV9nhcuy3FU6bm+X3FtKOru0279tPvtbQ55TnFux7bq3xj8KaPrraTM97LJFKYZ5ooP3cLhirBskMcYydoPHTPSqOn/ABNe4+Llx4eb99pE0SR2TwW7Mxk2B95PUowLfMAVwEYYXcx8q8T+Cr631XU7ez8DazBIsqi3azme5tlQKuSCYiz7vmOdy43AEDaQe50/T/FHg74h2esy+G5tRj1PTLazlWwCqLZwkCyZCjYuDGcDKoQRhhg4J5Zl9OjenrKUHZOUd/daatdLr1/zFzzb1Paa8L0PXZZU8XfFO5uLmf7MzWWl27uQEViNiyIpAKjzIuAx53tgtg17pXgng/SG1LwB41+H6TJ/bdrePKqqRtmKMgwm4g4Lw7SxAA3qfavKydU/ZVZT2vBP/A5e9+lzSpe6+ZjeL9T+I7eAbW913UoJtH1lAojWOIMu4bk3bUBG4LuGCemDg8V65rGrXHhL4PrfWyAXVrp0EUWCP3bsEjDcgg7S2cEc4xXjnjfWfFTeA9O0DV/C9zY22juqS3pifZIUUxx4bG0DB5ILBjgjA4r0PUx4t8Y6D4w8MS6J9mjt2RNMuGiaFLhY5s43O3zMyoMFRt9SuRXoYvC0Z1aU5qEbS95RslycyUXpptfztuRFvVK5z/hL4k+JG1CO41DxFpmr2i20k91YLEYJ4o0jMjMhMSK7rtxtDMDk9Bl1gn8Z/Em38K2vjVtZ0w6XcXJC2Plxhhh2GzBUMV+Qj5XLY57EiPQtC1fXfEHg+GHwS+hDRWjlvb6aAxC6CGMlmPlqSxKHAyxy56AE1h6j4J1fX/ED21l4J1DRrue8cO7OfsMKZbOD5eAAMHIcg4O1cFVHqxo4H2zvGC2buoOyTl2aSvo7pNpWTIvKx6BeXK+G/izoOvadf3MujeLlVZYi5cyOQAh2vgqoMkRHOVG8AAYWvX/SvHfiBa2mveKvCnw306fybODElzGrg+XGifIoY7mDiNZMAjB3oTnOR7FmvlM0s6VCb+JxfryptRb87aeiRvDdoKMUUYrxzQKMUUUAFFFGaACvOvje5/4VbqMQ6yzQIB6/vVP9K9Frzz4xn/ijbVdu7dqlqNv975+lAmegRoEjVR0AxT80AUEc0DCkoOc0Y5oAinghuraWCeJJYZVKSRyKCrqRggg9Qa4o/CDwL/0BB/4Fz/8AxddzjFL3rejiq9C6ozcb9m1+QnFPdFXTdNstI02DT9OgS3tIF2RxJ0A/mSTkknkkknmrdIAFGAMAdhSkZrGUnJuUndsYUmBnpRS9aQCHkc80lKBjg/hQDzQB5z8ZQz+G9GtxnFxrdrEcdcfMf6V6NxXnfxWHmDwdBu2iTxLZg4OD/F0/OvQyRkD1oEtxcen60d/akGOSBQNxBzgfSgYvBo4oxwPaigAHBxxQfzpNvpxS55oAOg4oySO1HccUntQAew470cY5NL9KTaCOeec80AJ3xzz7V5j8UXC+L/h3COjawHx9DH/jXqB+vSvNPH0CXHxN+HUTkbRc3cvzHHKrGw/UUhPY9IIUvu5yRj8P8mnZwBxnPpQM7jR+WKYwGOlOyCcelNyOn9KDnrjpQAccYpoK52jsKcBxxgenFIQMg45x6UABYY9MDnNJkdyO3NOx82c9vSm5zkjHpQA+jr7f1pOnOabn5sE/lQA7HQ57UYPr+tKaBjFAHPa5aRSeH9TXz2iQ2bEyy3UkUQ4PUg5UepHaq/hrS9P0zwnpmmtdx3y2luYw44D44bA9M8VV8eiCbwFrxkjikf7BPtGw/KRGec4PccE45xVvwPBDF8PPDqKpjQ6bA+BnqYwST+JoF1NEW6zNl7YpGdgGXDb+hz36dOeuPpVkwQbsSfMxBVM+/NS8B9yBs4PPYmiQZi5XO3BwMc/nQUMdNrCTyt8ioduAP544pQsjffIEeBx+eTnv2p6MoD4ccHnBzig8KCGGQOefb0oAdghRt+XHT0NI8hU/NsCg9+9PBBP97igH5jlB064oEY0mLfxdBtyq3WnyLJyMfunUr/6OkrZPJBPOBng96yNZcQ6hoTsF2m+MbEj+9DKB+ZxWuQByMc/lQAd87SOO/ag5zjHGOTSKVwTwDnB4xzUvU/zoAZuA4JAPpijOD/hScgepPGOlO6g4/Q0AIOOcV558XY45rPwnFIMo/iS0DD2xJmvQzgc/5Nef/FX73gxAeT4ls8f+PUCex6ARk9AcdMinZ9/yprAHIJ4/lTguCfQ0DDjNN6ZyD19aB1J5pfXjmgBenNA6c0fhzRj2oACce1KKaetKDkdMUABznHajJGPf3pcUd8d6AEyaWkx6fpS55x6UAFJjnrQc0cjGaAPMfhOFOu+PpQ2d+vTDHoNzY/nXp/X6V5h8JFDal45lxgtr84z+J/xr04A88igS2FqKaaK1t5J55UihjUvJI7BVVQMkkngADvUhGRisLxru/wCEF8QYIA/s25zkf9MmrSjD2lSMH1aQPRHlOpap8P8AUfHc/iMeNLqG3vIPIvrFLKbFwhj2FN+3hCAuRgnIJBBwVn8IeBNG1+eF9L8eahqOh6ZeCZNOVZIWhbJZOSwKnJPzqgz82CDnHBaJrFla6fpem6V4RtNY1y5B3TXUZdN/mOBHsIwRs2HdkdevGK9J+DEDW3iPxvBJBDbvFdxo0EJzHGQ83yqTztGMD2FfW18T7OlXp4eck6Vo68rVlLl/lTT1dne5gldptbkt18Fbq/lFvd+NdTuNLFyZxaTIXPLEk7i+3edzZfb1YnHOK6SD4df2f49k8R6Vrt5Y29zL595p8Y3JcSHdnJJxtJYnBUkZbaVyNvccUYzXg1M4xtRcsp6WatZWs99LeW+5qqcUV720g1KwuLK6j823uImilTJG5GGCMjkcHtXkXhDw7daho+qfDLxXYXKLYsLu2voFUoqM+RscrwWO8gnJIMinbtxXpnhvxPpfizTJL/SJHkt453gYvGUO5cc4PYgqw9mGcHIF3UtQi0nSr3Up1dobSB55FUAsVRSxAyQM4HrSoYivhebDuPvNpro4yWzX3teYNKWp594a+EP9j+I7DV9V8QTax/Z8QjtYJoMLHjhMFnbCrkkAYwcEHjm3onwvbSPA2seGT4huXXUWLiaKEReUcKDxklg20BgWwV4G3JJg0n4oyx+CpfFXiXT0tbGe8MOnR2bGSWVckYYHABG1vmJXO0/KON2x4P8AiVofjW/uLLTo7yG4hh80pcxqu5cgEgqzDgleuOoxnnHoYmeb2nOpqotXaUbJxd1sujetvRkRVPZG/oGh2PhzQ7XSNPRxbWylV8xtzMSSSSfUkk8YHPAA4rOs/B9rZePdR8WJcTNcX1slu0BxsXG0Eg9eRGnHb5uuRtr+MvH2leBvsX9qW95N9s8zy/syK2Nm3OdzD+8P1qrpvxQ0HUvCupeIlhv4bLT2CSia3+ZmONoUglSSWAxnjIJwCCeCFDHyg8RGLaqaN97vb5tfeW3G9uxw/ge+i8WfHTWNZnsJrVra1byIZ8rJEw2w5YDuR5mVOcE45wDXtmc9K8Q8IeONI1X4ua5qcAMMmq2kUFgl6REHlVQNjMu7buIGDz+eAe8+H3jS98Upqljq1glpq+lT+TdLCcxEksBt5JyCjA8kcAg84G2Y4bFzvUqU+SMFFW7R2Xrru+7Jg47J7naUUdqDgivGNQz+tBzkUyVPMjaPcy5GMqcEfSngCgAPFGf0oo7UAJnmlopM96QC5NFJ1BpRzTAM4+lHeiloA89+E774PGDjgHxNeH9I69BzmvOvhEQbDxWex8SXh/SOvRcDHT8qBLYD6igUUpoGJS80lAPtQAfWijnNHagBaQjvR1ooAXtTe/elooAM84rzv4sNmDweo6nxPZ4Hr9+vROnFeYfFRpG8TfD+3XO1tcjkIHT5WX+hNAmen5oooHIoGFBox70UAL2pKOhoHSgApe9J1HejOO1ABk0ZorP1nU4tF0W91W4DGGzgkmZVxlgozgZ7nFAGgc4oGfWs7Q9Wt9e0Sy1S03iC6iWVA4wwBHQ+9aPNAHM/EOcW/wAOfEbnodPmT/vpSP61zWsaheaN+z3Z3en3D29zHpNkiypwyhvKQ4PY4J5HI6jBrZ+KzAfC/wAQEnH+j4/8eFKnhqPxH8JrHQbid4BNptsnmoASjIqspweoyoyOMjPI6104OdOGJpzq/CpJv0vqRJN3SPAdS8Qa7pjtbv4x8Qtdm0trqNfOdY2EsaORuMufl344U5IPAHNfS/hy7udT8IaPeXE267ubGGaSTAG52RSTgcDknpXlV18A7i7ML3fi+Sd4YlijMtkWKRr0Vcy8ADOAK9i0rT4dJ0mz0+BnaG0gSCNpCCxVFCgnAAzgelevm2KoVqMYxmpy5m7qPLaNlZbK5NOLT2LYzjn9KXPNFJ15r581FzzWHoHhHRvDFzqVxpNr9nbUJVklRWOxcDhUXoq5LHH+0R0AA26K0jVnGMoRdlLdd7a6ishaKKQ9eKzGGQagvbSDUbC4srqPzLe4iaGVMkbkYEEZHI4J6VP9aXjrTTad0BkeHPDum+F9Gi0rTIfLgj5Zjy8rnq7nuxx/IDAAFR+LZfI8G63KSQE0+duOvEZraPIrnvHrhPh74kJ76XcD84mFVUqSqSc5u7e7ElYpfDC0+x/DPw7GRjdZrL/33l//AGauuxWB4GGPh94bH/ULtf8A0Utbwz1NQMXmigUnvigBaOh6Uc0f55oAO9L1pKXIoAKKTPNIQM0ALgA0H2o70UAcz8Q5BH8OfETHPOnzL+akf1qx4IGPh/4cHT/iV23/AKKWsf4sXCwfCzXnyQDCE+X1LquP1rc8IQPb+C9CgkGHi0+BGB9RGBQLqbXNLkUntR0oGLRScDjpRQAuKBSZzzS0AFFFJzQAtFIeaD70AFcF8aTj4Sa79If/AEfHXe4rgPjVx8I9bHqYP/R8dAHb2UYjsLdFAULEoAA4HFWajRdkSr2AAp/agELkUUnWloASgnC55oNBoA+QG8beK7u4up5PEuqo5Hm/JduisxYAqqhgB1JwBwB0x0+q/DF5caj4T0a9upPMubixgmlfAG52jUk4HA5J6Vz83wk8DzzyTPoMYaRi5EdxKigk54VXAA9gABXYwwxW0EcEESRQxKEjjjUKqKBgAAcAAdq97N8yw2LhGNGLTTb1UVZWWitv8zKnCUXqSUZFJRXgmoViS+EtFl8XW/ig2u3VYYmjEiMVD5G3cwH3mC5UE9jznC43MAnNFaU6s6d+R2urP0e6E0nueY/HXMvgCK2XrcajBF+eT/SvTRXnHxj+bRvDkZ6Pr9opH/fdej1mHUU0UnNL9KBmHpHhLRdD1nU9XsbXbfalKZJpXYsRnBZVz91S2WI9T6BQNyjnNGK0qVZ1Zc03d+fkJJLYD04oFFHesxgTRmjvRQAlLR3o70AHavO/jAw/4RzR4e8+t2kY+uSf6V6JXnfxVIkXwdbkf63xLZ/l83+NAmeiUc0Y4pMGgYUUuKTjpQAUUuMDFIaADNLSUvAoAQmilNNGTyDxQAufyoxRRg57UAea/FUbtX8CR88+IIDkdRgivSj04rzX4muG8U+AICeW1kSf984/xr0rjNAuod6QEntijGeMcUvWgYnI460uM46UdaP0oAOhxSYx34pfzoxQAzJ9OtOB5x+lAIPQ0ZHGOfegBTz0pBnGSMH0peoBpMZ6igAwck1574vijl+LPw8SRAwDai2GGeRCpB/MZr0E57/zrz7xTKG+MvgGMHlE1Bvzhx/SkI9CJxnPQUYB5xxR3wef6UE4/pTGGQcgHJHvTSGJGMDGc07I7c031xn1oAcD780jDIwCB9eaTI6ZOaARu5GPT3oAOCOmPXmlXAGDgnqccUvy5/CmhSCfmzznHpQAEDdnHJowcHpk96d1/wA9Kbz2HBH4UAO5Bo4pelLQBznjt9nw98QtxkabP2z/AMszSeCxu+H/AIcwT/yCrcf+QlqPx+zf8K78R/Lx/Z0/f/YOal8GH/igfDjNz/xKrfOR/wBMloF1Nx+QSRgA9zjNKeW5H05pSiOCGAO4d/SlC9CQCQMZxQMTOT2yR09aUgEjpTFXjHJxn5jinjOT8o56880AKAVHJz700jaM8nt1608+3H4U3nJHY/pQBieKWKaXAwPK6hZH/wAmIwf0rb75GMDrmsXxdj+wo+M/6fZcf9vUVbnHP+FACd+eKdkZB6U043Y3de1Ic8nt9KAHcflTeScjA9OadjuaMcUAH481558Uz/pfggeviW05/E16CRuHzCvPvij/AMf/AIHHb/hJLX+tAmegkkE9/ancDt1oIUk5GaOew/OgYAH8c0dCeaX6mgCgBBkjpj8aKWg4HWgAx/nNHGPaigjNABnimkbh3Ge4p3eigBBgnrR3paOAPSgAOaPY0c4oHU0Aea/B7DWniuTHzN4husn14WvSq81+DfOl+KP+xiuufwjr0rNAlsHfn14qC9tINRsbixuo/MtrmJoZUyRuRgQRkcjgnpU/tmjFNNp3Qzyr/hQnhX/n/wBZ+nnRf/G6830+zi8M/wDCwLjTNSubfUNIYWdkVnCu0LXHlSMQMbiAFGeilgcBtpH0L4q8QQ+FPDF7rU0DzrbKCIkIBdmYKoyegywyecDPB6V5Ho/i3QrjxrZXuofDhrGfXn8gXksrOkolAUssbIqENuXcy8kOTzuIP1+V47H16NSdW9SGnWO8WpNWbWjWjsno9jnnGKaS0OE8OT+IbHW45IPENnZSaxFMZLm41UbMmNvnmMbllcbyV3jO/wChp/g5tRsvHOi3Nxqrp/bE4inltLxJppVlI3LJsk3IWLDJbDKfmHzLXZfFHQ9L8BQWMnhvQHtJLhisuou5mj24OYdshYZYdcgZUMvzBnAr3mveA/Bl7p9xbeBrlPEEKxzy2tzdOFtWZdwBLFgWAKsPl43AnawKj21jPrNL2lGk5e0TSso30utfe0Wq77bK6M+Xldm9jZ+AFvpyWGp3K3v/ABNJZfLa1+0f8sVCkP5eefmcjcQcdBjJz2Pxg/5JbrIJ/wCeH/o+OuEvviP4E0jV4fE+jeGHudavlaSRpJVi8oFmRiQC4WQ7M8KCVfJPzEGv43+JF14l0nw//YsV/FbXzz219aQ7d0zlURoFOCWO2Tg7cfvEOCykL41TA4vEZnDGcjim0/eto46taN6aWTaRopRUHG5J4yFvFoPwpvdQh3aXBFCLt3iLxhCsBKsMHOVV+O4B4NT6z4l8Nx/HrStYg1GzNlbWL/bLuEgoZBFN/EPvttMajGT0XqMV1PgjwRf2/hi88OeK7SyvNJjkzp6yIplVWDFydpIVgXIBDEht+GK7SePg8B+GtR+NV14fh037Ppem2Immg8+R/tLkKQdxbcmPOXoT/q/9o4uhiMJJ1KU5NqEamsbWcZO/Xrra2193oJqWj72N/wAazeCPHc/ho6hrlzaWkq3MtvdCPyYZVBCshkkXCtuQEZ7KQQC6E+e63r3/AAj9r4k8GaPJ/bnhoxRPBNJN5v2YkxsXDx4G3zGxjgbtvqwappvgq48U+ENe8R2V0ljpunTzS22mu7yBQFV3G49CE2ANgliozjGa9f8Ahn4f8Pan8LoAdGhSLVIit8rOXM7xsU3FjyOVLADG0njnmt6ksNllFJylUjCSXK7e7K/MnfTVLtdXurpCV5vseP6BcWfhb4r6et/dWGtwQm2hN80+6GEsigOj5IIizgE8YXopwV9HTULfTv2kLlbeVEFzZpb3zXciIN5RCgh5GSSIRjk5L8Y5Hgv7u61D/lhZwyyf7ZjhBP8AwJtoH+8cDuak1KG6t9SnS8iSOctvZY1UId3zAps+XaQQVK/KQQRxivXqZQqsnzz1cJRelt3e9lZaeW7s355qpbofY+o61pejmP8AtLU7Ky83Pl/aZ1j34xnG4jOMj8xWPqXjfT9L8c6b4WuYnWa/gMqXDMqorEkInJySxVh9doGdxx8w6xFZ3EcN3H4ghvJ1sbYPE9tJE6uFEfkrhSreWqLliV3dsnNdPp/9iRa14H1TxBbONGfTnFxLcK0olkikmUAlVywBEQC4O1NinIHPz/8Aq1SpQ55ycnaWii078rasnZvb5+Rt7Ztn06PY15y/i7WdT+KNzpenXVna+H9DiMmp3MiiRJPlBZS/ARlOQBkY2OTuxtr0O3liuYI54JUlhlUPHIjBldSMggjggjvXjPhmznn1n4taOkeNRvfO+z20hCPIG8/awDY+U+YnPT5155FeHllGm41p1ErxSWvS8lFv5J/I0m3okTf8L35+2f8ACJ3n9j/afI+2+f8AjjGzbv287N/445r1+CeG5hjmgmSWGVQ8ckbBldSMggjggjvXzh/wm+i/8KJ/4RbfN/a3m7PK8v5dvn+dv3dNuPl9c9sc16NbeKbu20j/AIQXSIvs/i/T9IgCC6MflNIIoyyIdx3OFZiMjblST8oNelmeUxSXsaXI1KS1bs4q3vu+y11toRCp3dzZj+I+nXHxKPg6G1eRgrKbxJFKiZVLsmB2ABBOchgRt71z+q/GG6tNZ1iz03whe6jb6VK0dxcpMQE25DMwWNgq5VsEnkDPHIHl2jaN4t8IeP8AR7a20S2XXlgkkgt5ZlZZ1KygsxEm0ELuGAV+4OMk50vGXxBj8aapHo8VzDouhSyq99crG7/aJAoBdgqhnUbQEBAJwpbbwE745HhlXiqcFUp8ibfM97u8rRd3zJe6l1v2ZPtZW10Z6Jqvj7VNP8Q+GtbhuLWbwfrapCVdQhtHJG5pJRkBlyeM4wjjAK769QOc8V458TJfDz/CrRtO8PW0NzDeXMa6XFbOdwI3bmCfeduSjA87pMn5q9X0yO9i0qzj1KdJr5IEW5ljGFeQKNxHA4Jyeg+gr5/MKVNYenVjHld5Rs9G0no2u+tn1ujWDd2i39aKP84o/CvHNDzj4OEto3iNyCC2v3RII/3K9I615h8D5Hk8J6tPNw8ms3DN7khM/rXp2eKBLYBR3o7Z4oPrQMWkzRR3oAKBQKXPFABRnmg0lABj2owfp6UUtACYIGK848fjd8Qvh6mM/wCnTn8kWvRyT6V5342Bb4p/Dte3nXpI+kS0CZ6JRmg0ZAwPXigYdeKQjIxnH0paWgBOaB0pTSdTn0oAAaOtGKOtABx2ppAIKkAgjp607FJxmgBECooCgKBwABgU4DHc0UdRigDhfjFkfCjXsf3Iv/RqV1eiRmHQNOiYYKW0Sn8FFch8amx8JNbwcE+QP/I8dd6gAjUKMADgUC6jqSjr1oxQMKQ96XtRmgA4ooFFAC0Uh9KP50AHNGMdKUUUAJ2rlfiScfDXxEen+gy/yrq8VwvxhmNv8KNddepSNP8AvqVB/WgDd8GLs8DeH16bdNtgf+/S1t9c8VleF0KeEdGRhgiwgBHv5YrWzQCAj0z9KMfhRRQAA55HIozRS4oAKKKKAE70Cg8CkJx2zQAjEjpThSUoGKAPPvjWdvwk1rHcwZ/7/wAdd7HEsMSxoMKoAA9hXn/xuP8AxanVOeC8H/o5a9CVgyBlOQehHegXUfSUtJ3oGFLSHrRQAtFJ0pe1AAaSlo5oADiikFFABwa84+NDSy+DbLToAC2parbWoB6HJLD9VFekV558WebfwgB1Piay/wDalAnsehUopKWgYUUY70UAIaKWigAooooAMUUUUAFFFFAHnPxZxIng+2/jl8SWmB7Dd/iK9GrzL4nYk8ZfD63IJB1bzP8Avjaf616aOlAuoUUtFAxKKKKAA0UUDqaACjmjFFACdqXvRRigArzb4lxmbxX4AhHA/tgSf984NeknpXn3jj958Q/AEPc3dzJ/3zEDQJnoFKaBRQMMUCijrQAE4oooNAB3pO/UUY5zS0AJ3pTzRRQAmMcdqOTS0mRigDzX4gfN8Svh3FtDA3Vy2CM9Fj5r0qvO/FwEvxe+HsWfu/b34/64j/Cu/RMO7GRmDEYB6L9KBIlo6dTQfpS9qBiZ4GKB34xQKMc0AHeg/WjpR9KAA59cU08jCtinUe9ABg456UmBjgU6mE5OB2HpQApGex49K858SPu+OXguPj5LW8f84yP6V6PjkcfjXmOvNn9oXwsvZdMnP5iX/CgTPTjz/wDrpu3kjoD6U7nPOMUHrQM5Tx/40g8FeHZbv9zJfS/JZ28jH94/GTgc7VByenYZBYVHZ/Enw1L4WtNfvNTtrWKdQHhLl5EkG3fGFA3MVLDOF6EN0INVfi7ZG9+GWq7bbz5IPLmT93uaPEi7nHphC+T6Z7ZrxDxLDa6jpXhTVPst5ZaImmpYS3MVmG/0mNpC+FLKG3Md27cM5bqysB9PleV4XG4aDndPmabXblvZLz6b9fQxnOUZaH0LN4+8KW2jR6tJr1mLOT7jK+52Py5XYMtuG9cjGVzyBXPeKPitpmk+FLPWtDktdTW5uxAIjIY22rzIdpG4EDA5HHmKeQQD4adJsk8J2t7eHX4rKXU5kt7sWyNbmLyxkiMuMSsyqD823CEAsUIqex0i6v8A4d6/JpthPcWlpqUE7XZjKu8SxzA7l3Ffl3oxC5K+YSSQAR6dPh7A02pyk5JStrorXta/e++vlbqZutJ6H1FpupWmsabb6hp1wlxaTjekqDgj+hByCDyCCDzXA/EjWNXu9f0Hwb4f1F7O71JjLdTQ5WWKEHhlbIGMLISAdx2AcA4PX+Ede03xH4ctr/SbWa1shmGKKWDytgT5cKB8pXjjaSO3UEDhvFf/ABLvjx4R1O8/d2dxbPaRydd0v71duByOZo+SMfN14OPnsvoqGMmpR1gptJ66pOya623+RtN3iQar8QvF0niPU9H8JaTDq8GjxBLq5uImMjyLw5wpQbtwICqCWKkrkcDtPAPi1fGXhaDVGRI7lWMNzFHnaki4zjPYgq3fG7GSQa8zTxJL8LPHPi59W0q5nh1edrizmiyscjAs4XcwGRiYBiM7SOhzSeA/EVx8PvCvh+3vdNeZfEWoSSoUZw8Mf7mMN5YQlyeWAXqNuOvHqYvLY1MNahTV/d5WnrP3W531tpbsvLsRGdnqxutfGjxPYeLNQ0e0stG8u3vpLWJp1deFcqCzGQKOnJOB9K7/AMT/ABR0rwbfW2n6zZXpvJbZbhhZhZI1yWUgMxUnlTztHGPpXnHiHxd4Zto/E+l654NhtvEk0tygnhtkkTey4jlDybWXPytlV5++BliKy9V+HHjfWdI8OyJpU0rwaYIZPOuI1eP99KyIQ7AjEbJx26cYwOt5dgansniIKlHbVpc2l7p3tb/Mnnkr21PaviK3l/DfxEzNj/QJRnHquKt+CiP+ED8Okf8AQLt+P+2S1nfEwM3w01/EYc/Y2+Vu3qfw61o+CxjwJ4fGCD/ZluMHr/qlr4c6Opt88cdOtHvg/gaFAXj0rz/S/itpWqfEK58OrJbLY7Fjs70SHE84+8o4xg5wpzglOC29QOihhK2IU5Uo3UVd+n9fqDkluehcUdO/1rnLXx74UvdaOk22u2cl5xtVX+RycYVH+6zHcOFJPXjg1HD8QvCVzriaPb67bS30rBIwm5o3YjIAkA2EnpjPXjrxT+pYnX93LRX2e3f08xc0e5027n17UvJH9c1wfhL4lWPibxVrOiP9miaCdlsGjl3/AGuNchmBxgn5d3B+63Q7Sx7W9u4dN0+e9upClvbRNNK+CdqKCScDk8A9KWIwlbD1FSqRtJ2/Hb+u+g1JNXRi+Kka4/sWyjGTc6rAS2egizOfzEOPxrfAYZ7jPevnbTfG+tQi88Za1dPdOoLadYs7C3jnfdEhCqTtARbnIO0nZySWBrs9F+Iviy28V6RpfjDRLXTrbVgBbyxxOrb2+6D8zc5IUqcFd4JwOvo1MjxEeblafLfru0ryST1dutiFVR6zxRjjpXEfEzxfqPgvw5balp8NrLNLdrAy3Csy7Sjt/CwOcqO9YvgH4lax4h0nXdW1m0sEsdLgMp+xMRMSFLEeWzHIIHDEqMjAzzt56eV4iphfrUUuW9t9b3sNzSlynqHToeabjOeOa8Y8NfFXxfq9/YtJpGjXdpcShGt7K5RbsjO0lY2mLcfeOVA2gklR8w3PDmqa14e+KuoeFNZ1aa+s7+Jr3T5bkBpCepUbeFUBZBjAGYwVC7sHatk1ejzqclzRV7J3ulvt2316ejEqiZ6Z1OCP61538Uj/AMTLwKPXxHan9a9FJPHFedfFI41fwIM/8zFb8fjXkFs9Fxz3zRx3FBI59utGc+9IYY9KXmjGaT6UwF+lGcjnmjr0xScUALSfWgfWl60AAOelB/WlwAcij3oATkjpQfTg0tIetACHnrQO4psi7kKkkZ7qcGhQQAM5AGMnqaAPOPgyQ2k+JmAwD4hu+Pwjr0oAY/xrzX4M/wDIC8Rt6+ILo/pHXpPpQJC5paToaWgZyPxP0y91b4davZafbPcXLpGyRRjLMFkVjgdzhTwOT0GTXhnhjw/43vvGfh59S07WDbWN1Bsa4tnjjt4o2XPLAKMKgHqdoHJwK+oOtBAYYIyK9bBZq8LR9lyJu7abvo3Hle2+hnKHM73OD+LPhfVfFXg6Gz0mJJ7qG8SfymcIXUK6kAnjPzg8kcA98A8J4o+H3i7U9fTxFN4e0zU7jULaP7VYm6ZEtZVVF4IkQtkLnhiBlhzgM3K/FiWS4+Lt1bzi4uYhJbQJCkmG2tGhKxlshcliRwRkk4616h8Bp5ZPAVykkrukWoSJGrNkRrsjbA9BlmOPUk969mnUq5fgo1KU03FJtOLWlRXtdS/urZJ6b20M2lOVn/Vjj7j4YeKbPR9EhXwxoeqtHBKZ0DmGVHdwwErrKnmFRgKQcDLDBwrG1afDXxlZ+EdDukSGTVtH1OS7t9OmmDDy2MRA3bgow0ZYqDghychuD7uKOorz3xHi2kmo7t7Pre63tbVrSz8y/YxKWjS6lPotpLrFtDbai0QNxDA+9EfuAf6c46ZbGT5jqd3b+DPjyNU1GTZp+u2Ih+0yApHAw2rjdyG5iTPTaJQTwMn1vjvVLVdG03XLVLXVLKG7gSVZljmXcA6nIP8AQ+oJByCRXn4PFwo1Zucfdmmml0T7X7Oxco3Wh4zL4L+InhfTda8NeHba2vtD1JnZZTLH5saNlSpLlPmZAobggfwkHNdVoWg+MvCureGdH04pP4ct7PGolpIgvns0jSFSV8wgFl2gAA4AJHzGvSqT0rprZ1WrQcJwi73vpu7Wu9d0tmuupKppbM+RDpt5Y33ifw7Zw2l75Bk82aYKkipbOxMkYZuGxnIG47SQO9dl4bg8XarpFvf6d4d0PxHZGCO3T+0xBNJZmJdhjGShUHAcLyMODkszE42s+Cdc1v4j+KIdL06LUJre6eSTE4jEYnJZD8zLk4PTkZHOR1ueAtQ1/wAD2vjDUYlttmmLHBeWcw3F5zIY4yGU9EO8nBwRx3DL9fKt7ehOVFwlK8Wtb3cuVO9n7rctFt2fU50rPW5a1zw5aeDvhxDoF9Z2V54u1i5SSKOKIPcWsZK/KrAEtkptwCAS7Y3BST7bpXg7SNP8Kaf4fubK2v7WzUHFzCHVpOS0m1t2CSzHrxuwOK8H0P4ma9f+Mf7SuNKttW1IwTx2Sw2O+WDKOyqmwhiu7GSxZgm/BG5s6fhH4teMNV8ZW1lcXVlLBfymFIZYkjjgLH5WU5Vm29lLEsPlB3EEcOY5dmNalZyScbzk+bdvtpoklbW3UuE4J/gfQUU8VwheGVJEDMhZGBAZSVYcdwQQR2IIrhdd8IxWvjuw8YWWuJpEjNs1FZnGy5hSMsQMnGdsfI6ALvGCnzcz+z/FqQ0LU5muYTpZudqQbP3gmCqWbd2XaUGOckfw4O7D/aAi1JdZ0iW4uYX054pBawom143GzzCx/izlMHjpjAwS3lYTLpUs0lgoVbXTTdr3Vr2s9P00uXKd4czR6No+u+BvFH27xGun2cf2G5VH1O/s0iywwEdZWH+7jJDD5cgZGeg0mbw3qWpXOo6RLpN1fbVS4ubRo3l2noHZecfIMAn+H2r5a1fxjd6n4X0zw3FbQ2ulafh1jTLPJLtO52Y+rNIQBgDfjnANTnXtS8Ka+NT8P2s2h/bLGLbHJBuDIyoXZPN3ko0iMVOTx37V6tThmc01Gbi3flTd1ZW0b897JNL5awq3kfUmp6loukzwT6pfafZzMrpDJdTJGxXKlwpYg4yEyB6LntWO9l4AvrW51l7bw1cW4lP2i9aOB08wkZ3ydNxLDqc/MPWvCPGuo6l4u8TeGL6ezs5rvULGARWcUn7tiZpE2M4f+JgSeVKhtp5Uset8A6Bo2oeINc8KeI/DEdnfrBFO9vBdyNAFUghv9YxEn70fMGPykj5ctv4JZPHC4ZVZVZKSV2o22UrO2qbt32uV7TmdrF/UrjwzdfFjSHm1p9UsLaBW0vTtIhM0Vm6DPzCLJIygYBQT0DbUUbu78OfEXwz4ltYpLbUoLWeWXyVtLuVI5y+cABc/NnIxtz1x1BA8S8L6HbjxX4x1nS1Q2Ph+C8uLCVGSWNZBv8g/Nu3gBWYHnlFOfXhPs1rBZ+ZcT+ZLcW3mW627g+XIJtpWYHp8iuwA5+ZD0Jr1Z5Jh8WlSdSV4KKW2l7vVLyabd7/rmqjjrY+zp5YraCS4nlSKKJS8kkjBVRQMkkngADvWXD4u8N3M8cEHiHSZZpWCRxx3sbM7E4AADZJJ7VBpcMXinwDpya3El4uoafC9yrqAHZkVieMYOeQRjBwRjFeQv4U8Nah8YrbQdC0xF07So2n1FhMZRI687TvdgVDGNCoAOS4PTI+XwWBoVfaxrSacE3olay9Wnq9ErG8pNWt1Nr4K+JNFsPAki6lrWnWl1NfSytHcXSRtzjnBOccV6Bc+N9Fs/GMPhe5eaC+niV4pJYysUjE4CKx6sccYGM/LndxXzNptx4Xg8DXUOo6Pfvrlwxk0+7Rykax5CjOWwQGWQH5TnkZB5HoviL7VL8FfCHiOTybLVtIlj+ytJlWaMEqmxGyHYhIpORghWI44Pp/2FQj7NuTam+VPS12rqS3vG+nQzVV6nu5xxR2qrpmoRatpNnqUCusN3Ak8ayABgrqGAOCRnB9atd6+WlFxbi90dAUYFLmikAh7UHPal70lAC0nvS0dqAEyMZooAAGAKKAAmvPfGZI+LHw7x/f1D/0StehGvO/FQz8ZvAHIOEvyV9P3PX/PpQJnohI+lIACcgAn1pcDOcUtAwxRkUUn1oAOaKXr9KQYHFABz3HNHalo/CgBOfajpRS8GgBKODS0mBQB5r8dXYfDSaJf+W11BGf++s/0r0uvNfjUf+KW0mLGRNrNtGw9R8x/pXpJwMc0CF7UnbBoH1oB9qBi0nGfrR70fjQAopKDntR3oAMij615J8TvG/iHQPGOgWWmWV4tssolITBXUSSFMS4DHgEjHXLg7eEYz678cdK0fWRp0ekXk5hl8u9Z3VDCwxuVQMh2U7geQMrwxBzXrQyTGVYU50o83Om9GtLPr/XluZupFNpnqtHWvI9b+POlafLDFpmkzX++JJJGe4WJU3IrBQV35YbirDjBUjmqt58TdRvfiR4bk0KDULrR7yzH+gKqK05ZnV26nBQpjLEAeW2CFYsahkOOa5pw5VZu7a6K9vJvpe3cPaxPZq82+OWoWtt8MdRs5biJLi6aIRRM4DyBZUZto6nHGcdM16TXzF8Qv+Kk1jxrrFw8i/2XcwafbwM5YL+8KFgcjAPluduMZlPcZPLgsGsQpyk7KK+9tpRXzb3HOVrH0pZ2y2dlBaISVgiWME9cAY/pVjBIr5y2+OP+EB/4WB/wmN5/x8+Z9k859u3zdmdudn3/AODbt29/4a9qvNRutX+G1xqdhFNFeXmkNcQRwMWkSR4SyhSACWBIwQM5roxeVPDuNqiknJxdr6SVrrX1FGd+h0dFfN/gjWvEtj4m0nUPFOteIrLRZmHl3F0ZGtpmZSUVmk+UKwyd2DjqNv31g8T+Mb+bxzr6XnifXNLhgvHggh0wM8e1CUyVMyBThQTjOSSeK7/9WqrrukqiaSvdJvra2m/n26k+2Vr2PpEXtp9v+wfaYftnled9n8weZ5ecb9vXbnjPTNT5rw/xdE9no3hP4kW1zDqGo28sQ1C605GiS7Tplj/BjaYiSozvwQuAg9st5YrmCOeCVJYZVDxyIwZXUjIII4II715OMwSoU4VIu6d09LWlF6r8mti4yu7ElFFFcBYmRRgdaWigBOKOvUGiigDzf43OT8PfsijLXl9bwKPfdn/2WvSK8++KgDr4OjPIfxPZAj1Hz16D3xQJB/KgA0uKKBiHil6UcUhAPUZFAC5zRRQc9qACijmigAFAoooAOled/FRgZPBUWRlvE9mcf99f416J+FeafEndceNPh9p46PqpuT/2yCn+tAmel8UUnfpS9aBnH+I9a1bT/G/hLT7JGexv5LlbweXkYVAV+btj5j74rr+opjozFMNtAOSMdR6U8elAC54o4phRWUq3zA9Qaf2oAKO1FFABRSGlFABR3oooA858dxiX4l/DyM/8/N2/5Rqa9Grzzxfh/i78PUJHH9oHH/bEf4V6FQJbi0UtJ0oGFBpaSgAooFHWgAo+lFFABSc9zS0UAGOK888VzK3xh+H8CsCyrqDsvoDBgH9DXofavNdaiEvx+8MknmDS55B+O5f60CZ6VxR7UcUUDCijNFABRS0lAB9aOM4pCcUvWgA5o75oyKTHtQAvekpTzSGgDzbxCN/x38HLn/VWV2/5owr0nivNdUbf+0HoURHEeiyyD2yzD+lelcUCQdqWkooGGRnjrR9fxpe9IQDQAUUYweKCD1oAAAOPT1oxzmgkZxij+VAC0lBpMZ7GgBfSvM75Ym/aJ00SOVKeHy0a4B3t5sgx7cZPHpXpn4GvPNqyftCAtgmPwxkex+0//XoEz0OkyMjv/Sjv8uMGjjIJHPagZ5d468QeLG+Iek+FfDGo21i11aNP5k0asGb94SGJVsACPjA6k57YzPDPijxpY/FS28L+ItWtr9JUk80RQKAhCM4KkIpz8g9RhvXpD4+1y18M/G3Q9Xu1cwQaad2wDJLeeo/Vhnr361maJqtpr3x90rVLS8guftMUjSCCORUiZYJF2ZkVS3yqp3bRnPQV9fTw/wDsqXsU4eylJy5deb3vtW326nO372/U995JGVoP3cYNQ3FzDZ20tzcypFBGC7uxwFA6kmiCdLm2jniJKSKHXIKnBGRweRXyB0E/0rm/GfgzTvGujGyvVKTxktbXSKC8Dnv7qcDK98diAR0RwT3JHOKTA3k4IJ4JrSjWqUaiqU3aS2Ymk1ZkVlb/AGGxtrUzTXBhiWPzZ33SSYGNzHuxxkn1qwRyOB70n059KUDnJ61Dbbuxh3o4oIGeRRzSA4r4sOY/hdr7Ahf3AXn3dRW14SJPg3QySuTp8HKjAP7sdBWJ8W1D/CzXgQD+5Q4Jx0kU1ueFgP8AhDtEAPH2CAAg5/5ZigXU1+AMk8D1rwjXLWK1+MniewXSnafV9Klh04R24wZ5IFzID2BIlVnHAJbcQNxHs3iDUZdL8NapqECo01rZSzxhwdpZULDIBBxketePaZqPxT1XwrB4iTxRp0Omyh2d7iKJTCqMwLN+66ZTHGTyOK9/JVKlCpXcoqLXL7za1eq2T7GdTWyPN9D0lJdd0uyhOs/2yL5UntLe2WKSEKx3GOQvkOoGfmVQpyScLkwXVlp0OpiCwh1O4vFvjENMvbTaSgchUZkk3FzhQVCryTg8DPufwo8W674gutdsdbvY7yWwkURypD5bNksDxhRj5BjIDc/gPT9vrz6Z7V7WL4krYXESpzheyW0tNdf5VpZrs/MyjRUldM8</t>
   </si>
 </sst>
 </file>
@@ -461,10 +518,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -495,135 +552,138 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="F2">
         <v>207</v>
       </c>
       <c r="G2" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="F3">
         <v>207</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="F4">
         <v>207</v>
       </c>
       <c r="G4" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="F5">
         <v>152</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="E6" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="F6">
         <v>207</v>
       </c>
       <c r="G6" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="H6" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="I6">
         <v>5</v>
@@ -632,33 +692,385 @@
         <v>202</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="F7">
         <v>207</v>
       </c>
       <c r="G7" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="I7">
         <v>5</v>
       </c>
       <c r="J7">
         <v>202</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8">
+        <v>69</v>
+      </c>
+      <c r="G8" t="s">
+        <v>44</v>
+      </c>
+      <c r="I8">
+        <v>11</v>
+      </c>
+      <c r="J8">
+        <v>58</v>
+      </c>
+      <c r="K8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9">
+        <v>69</v>
+      </c>
+      <c r="G9" t="s">
+        <v>44</v>
+      </c>
+      <c r="I9">
+        <v>11</v>
+      </c>
+      <c r="J9">
+        <v>58</v>
+      </c>
+      <c r="K9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10">
+        <v>69</v>
+      </c>
+      <c r="G10" t="s">
+        <v>44</v>
+      </c>
+      <c r="I10">
+        <v>11</v>
+      </c>
+      <c r="J10">
+        <v>58</v>
+      </c>
+      <c r="K10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11">
+        <v>69</v>
+      </c>
+      <c r="G11" t="s">
+        <v>44</v>
+      </c>
+      <c r="I11">
+        <v>11</v>
+      </c>
+      <c r="J11">
+        <v>58</v>
+      </c>
+      <c r="K11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12">
+        <v>69</v>
+      </c>
+      <c r="G12" t="s">
+        <v>44</v>
+      </c>
+      <c r="I12">
+        <v>11</v>
+      </c>
+      <c r="J12">
+        <v>58</v>
+      </c>
+      <c r="K12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13">
+        <v>69</v>
+      </c>
+      <c r="G13" t="s">
+        <v>44</v>
+      </c>
+      <c r="I13">
+        <v>11</v>
+      </c>
+      <c r="J13">
+        <v>58</v>
+      </c>
+      <c r="K13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14">
+        <v>69</v>
+      </c>
+      <c r="G14" t="s">
+        <v>44</v>
+      </c>
+      <c r="I14">
+        <v>11</v>
+      </c>
+      <c r="J14">
+        <v>58</v>
+      </c>
+      <c r="K14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15">
+        <v>207</v>
+      </c>
+      <c r="G15" t="s">
+        <v>44</v>
+      </c>
+      <c r="I15">
+        <v>5</v>
+      </c>
+      <c r="J15">
+        <v>202</v>
+      </c>
+      <c r="K15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16">
+        <v>207</v>
+      </c>
+      <c r="G16" t="s">
+        <v>44</v>
+      </c>
+      <c r="I16">
+        <v>5</v>
+      </c>
+      <c r="J16">
+        <v>202</v>
+      </c>
+      <c r="K16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
+        <v>32</v>
+      </c>
+      <c r="D17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17">
+        <v>207</v>
+      </c>
+      <c r="G17" t="s">
+        <v>44</v>
+      </c>
+      <c r="I17">
+        <v>5</v>
+      </c>
+      <c r="J17">
+        <v>202</v>
+      </c>
+      <c r="K17" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" t="s">
+        <v>40</v>
+      </c>
+      <c r="F18">
+        <v>207</v>
+      </c>
+      <c r="G18" t="s">
+        <v>44</v>
+      </c>
+      <c r="I18">
+        <v>5</v>
+      </c>
+      <c r="J18">
+        <v>202</v>
+      </c>
+      <c r="K18" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>